<commit_message>
[ADD] Continue label table editing
</commit_message>
<xml_diff>
--- a/data/Suspension Data Labeling_We_Re_edit.xlsx
+++ b/data/Suspension Data Labeling_We_Re_edit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GITHUB\Drop_wall_impact\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vulf/Git/Hub/Drop_wall_impact/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF7B4CD-0D6C-4C5B-92F1-A0225CE9B385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA535CBE-B201-0B45-B4BE-3F43E7450248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21600" yWindow="19460" windowWidth="21600" windowHeight="18940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Labels" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="69">
   <si>
     <t>Test #</t>
   </si>
@@ -118,9 +118,6 @@
     <t>*Разлетается больше чем 5 капель. Ближе к splashing, чем к semi-splashing</t>
   </si>
   <si>
-    <t>*Верно!</t>
-  </si>
-  <si>
     <t>*Брызг нет!</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
   </si>
   <si>
     <t>gear</t>
-  </si>
-  <si>
-    <t>* Несколько крупных (порядка 5), множество мелких. На виде сверху есть как отдельные капли, так и несколько "зубьев шестерни"</t>
   </si>
   <si>
     <t>*Образовалась "шестерёнка" на виде сверху - некоторые капли даже отделились, другие образуют "зубья". На виде спереди не видно отлетающих капель</t>
@@ -206,12 +200,77 @@
   <si>
     <t>* На виде спереди нет вылетающих капель, однако видно много частиц, остающихся после сбора капли. На виде сверху плохо различима капля из-за текстуры подложки. Однозначный вывод сделать не удаётся</t>
   </si>
+  <si>
+    <t>*Брызг и зубьев нет! На виде спереди остаются частицы на подложке. Однако на виде сверху виднеется один гипотетический "зуб".</t>
+  </si>
+  <si>
+    <t>*Брызг и зубьев нет! На виде спереди остаются частицы на подложке. Вид сверху плохо интерпретируется</t>
+  </si>
+  <si>
+    <t>*Брызг и зубьев нет! Однако на виде сверху виднеются разрывы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Есть как крупные капли, так и сохранение частиц на подложке при сборе капли </t>
+  </si>
+  <si>
+    <t>particles</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*Множество капель мелкого-среднего размера! Также, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gear</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> на виде сверху!</t>
+    </r>
+  </si>
+  <si>
+    <t>* Несколько крупных (порядка 6), множество мелких. На виде сверху есть как отдельные капли, так и несколько "зубьев шестерни"</t>
+  </si>
+  <si>
+    <t>*Две капли отделяются!</t>
+  </si>
+  <si>
+    <t>*Капля отделяется и возвращается!</t>
+  </si>
+  <si>
+    <t>*Отсоединение при отскоке!</t>
+  </si>
+  <si>
+    <t>*Небольшая частица осталась после сбора капли</t>
+  </si>
+  <si>
+    <t>* Одна-две капли отделяются при распространении капли</t>
+  </si>
+  <si>
+    <t>* Три крупные капли всё-таки вылетают! А на виде сверху следы и того большего числа - порядка 6 брызг</t>
+  </si>
+  <si>
+    <t>* Одна отсоединённая на виде сверху крупная капля</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,13 +316,50 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri (Body)"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -293,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -311,6 +407,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,21 +715,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K402"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.5" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" customWidth="1"/>
-    <col min="11" max="11" width="30.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.5" customWidth="1"/>
+    <col min="11" max="11" width="30.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
@@ -660,7 +761,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="315" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="192" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -690,7 +791,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -701,7 +802,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -733,7 +834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -765,7 +866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -797,7 +898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -832,7 +933,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -864,7 +965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -899,7 +1000,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -934,7 +1035,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -969,7 +1070,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1001,7 +1102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1033,7 +1134,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1065,7 +1166,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1097,7 +1198,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1129,7 +1230,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1161,7 +1262,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1196,7 +1297,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -1231,7 +1332,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1266,7 +1367,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1301,7 +1402,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1333,7 +1434,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1365,7 +1466,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1397,7 +1498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1429,7 +1530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1461,7 +1562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1493,7 +1594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1504,7 +1605,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1528,7 +1629,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1563,7 +1664,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1595,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -1627,7 +1728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -1659,7 +1760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1694,7 +1795,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -1726,7 +1827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -1758,7 +1859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -1790,7 +1891,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -1822,7 +1923,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -1854,7 +1955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -1886,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -1918,7 +2019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -1950,7 +2051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -1982,7 +2083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -2014,7 +2115,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -2046,7 +2147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -2078,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -2110,7 +2211,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -2142,7 +2243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -2174,7 +2275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -2206,7 +2307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -2238,7 +2339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -2273,7 +2374,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -2305,7 +2406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -2337,10 +2438,10 @@
         <v>1</v>
       </c>
       <c r="K53" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -2372,7 +2473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -2404,10 +2505,10 @@
         <v>1</v>
       </c>
       <c r="K55" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -2439,10 +2540,10 @@
         <v>1</v>
       </c>
       <c r="K56" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>55</v>
       </c>
@@ -2474,7 +2575,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>56</v>
       </c>
@@ -2506,10 +2607,10 @@
         <v>2</v>
       </c>
       <c r="K58" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>57</v>
       </c>
@@ -2541,7 +2642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>58</v>
       </c>
@@ -2573,7 +2674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>59</v>
       </c>
@@ -2604,8 +2705,11 @@
       <c r="J61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K61" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>60</v>
       </c>
@@ -2637,7 +2741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>61</v>
       </c>
@@ -2669,7 +2773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>62</v>
       </c>
@@ -2701,7 +2805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>63</v>
       </c>
@@ -2732,8 +2836,11 @@
       <c r="J65">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K65" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -2765,7 +2872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -2797,7 +2904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -2829,7 +2936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>67</v>
       </c>
@@ -2861,7 +2968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>68</v>
       </c>
@@ -2893,7 +3000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -2924,8 +3031,11 @@
       <c r="J71">
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K71" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -2956,8 +3066,11 @@
       <c r="J72">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K72" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -2989,7 +3102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>72</v>
       </c>
@@ -3021,7 +3134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -3053,7 +3166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>74</v>
       </c>
@@ -3085,7 +3198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -3117,7 +3230,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>76</v>
       </c>
@@ -3149,7 +3262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>77</v>
       </c>
@@ -3184,7 +3297,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>78</v>
       </c>
@@ -3216,7 +3329,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>79</v>
       </c>
@@ -3229,14 +3342,14 @@
       <c r="D81">
         <v>0</v>
       </c>
-      <c r="E81">
-        <v>1</v>
+      <c r="E81" s="8">
+        <v>2</v>
       </c>
       <c r="F81">
         <v>1</v>
       </c>
-      <c r="G81">
-        <v>0</v>
+      <c r="G81" s="8">
+        <v>1</v>
       </c>
       <c r="H81">
         <v>0</v>
@@ -3247,8 +3360,11 @@
       <c r="J81">
         <v>1</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K81" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>80</v>
       </c>
@@ -3280,7 +3396,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>81</v>
       </c>
@@ -3312,7 +3428,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>82</v>
       </c>
@@ -3344,7 +3460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>83</v>
       </c>
@@ -3376,7 +3492,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>84</v>
       </c>
@@ -3408,7 +3524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>85</v>
       </c>
@@ -3440,7 +3556,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>86</v>
       </c>
@@ -3472,7 +3588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>87</v>
       </c>
@@ -3504,7 +3620,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>88</v>
       </c>
@@ -3536,7 +3652,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>89</v>
       </c>
@@ -3568,7 +3684,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>90</v>
       </c>
@@ -3600,7 +3716,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>91</v>
       </c>
@@ -3611,7 +3727,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E93">
         <v>0</v>
@@ -3632,10 +3748,10 @@
         <v>1</v>
       </c>
       <c r="K93" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>92</v>
       </c>
@@ -3667,7 +3783,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>93</v>
       </c>
@@ -3678,31 +3794,31 @@
         <v>1</v>
       </c>
       <c r="D95" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E95">
+        <v>2</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H95">
+        <v>0</v>
+      </c>
+      <c r="I95">
+        <v>0</v>
+      </c>
+      <c r="J95" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K95" t="s">
         <v>35</v>
       </c>
-      <c r="E95">
-        <v>2</v>
-      </c>
-      <c r="F95">
-        <v>0</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H95">
-        <v>0</v>
-      </c>
-      <c r="I95">
-        <v>0</v>
-      </c>
-      <c r="J95" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="K95" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>94</v>
       </c>
@@ -3713,7 +3829,7 @@
         <v>1</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E96">
         <v>0</v>
@@ -3734,10 +3850,10 @@
         <v>1</v>
       </c>
       <c r="K96" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>95</v>
       </c>
@@ -3748,31 +3864,31 @@
         <v>1</v>
       </c>
       <c r="D97" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97">
+        <v>0</v>
+      </c>
+      <c r="H97">
+        <v>0</v>
+      </c>
+      <c r="I97">
+        <v>0</v>
+      </c>
+      <c r="J97">
+        <v>1</v>
+      </c>
+      <c r="K97" t="s">
         <v>37</v>
       </c>
-      <c r="E97">
-        <v>0</v>
-      </c>
-      <c r="F97">
-        <v>0</v>
-      </c>
-      <c r="G97">
-        <v>0</v>
-      </c>
-      <c r="H97">
-        <v>0</v>
-      </c>
-      <c r="I97">
-        <v>0</v>
-      </c>
-      <c r="J97">
-        <v>1</v>
-      </c>
-      <c r="K97" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>96</v>
       </c>
@@ -3804,7 +3920,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>97</v>
       </c>
@@ -3836,7 +3952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>98</v>
       </c>
@@ -3868,7 +3984,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>99</v>
       </c>
@@ -3900,7 +4016,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>100</v>
       </c>
@@ -3932,7 +4048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>101</v>
       </c>
@@ -3964,7 +4080,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>102</v>
       </c>
@@ -3996,7 +4112,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>103</v>
       </c>
@@ -4028,7 +4144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>104</v>
       </c>
@@ -4060,7 +4176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>105</v>
       </c>
@@ -4092,7 +4208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>106</v>
       </c>
@@ -4124,7 +4240,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>107</v>
       </c>
@@ -4156,7 +4272,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>108</v>
       </c>
@@ -4188,7 +4304,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>109</v>
       </c>
@@ -4220,7 +4336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
         <v>110</v>
       </c>
@@ -4252,7 +4368,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>111</v>
       </c>
@@ -4284,7 +4400,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>112</v>
       </c>
@@ -4316,7 +4432,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>113</v>
       </c>
@@ -4348,7 +4464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>114</v>
       </c>
@@ -4380,7 +4496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>115</v>
       </c>
@@ -4412,7 +4528,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>116</v>
       </c>
@@ -4444,7 +4560,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>117</v>
       </c>
@@ -4475,8 +4591,11 @@
       <c r="J119">
         <v>1</v>
       </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K119" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>118</v>
       </c>
@@ -4508,10 +4627,10 @@
         <v>1</v>
       </c>
       <c r="K120" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>119</v>
       </c>
@@ -4543,10 +4662,10 @@
         <v>1</v>
       </c>
       <c r="K121" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>120</v>
       </c>
@@ -4578,10 +4697,10 @@
         <v>1</v>
       </c>
       <c r="K122" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>121</v>
       </c>
@@ -4592,16 +4711,16 @@
         <v>1</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E123">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="E123" s="8">
+        <v>2</v>
       </c>
       <c r="F123">
         <v>0</v>
       </c>
-      <c r="G123">
-        <v>0</v>
+      <c r="G123" s="8" t="s">
+        <v>11</v>
       </c>
       <c r="H123">
         <v>0</v>
@@ -4609,14 +4728,14 @@
       <c r="I123">
         <v>0</v>
       </c>
-      <c r="J123">
-        <v>1</v>
+      <c r="J123" s="8" t="s">
+        <v>11</v>
       </c>
       <c r="K123" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>122</v>
       </c>
@@ -4648,7 +4767,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>123</v>
       </c>
@@ -4680,7 +4799,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>124</v>
       </c>
@@ -4712,7 +4831,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>125</v>
       </c>
@@ -4744,10 +4863,10 @@
         <v>1</v>
       </c>
       <c r="K127" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>126</v>
       </c>
@@ -4779,10 +4898,10 @@
         <v>1</v>
       </c>
       <c r="K128" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
         <v>127</v>
       </c>
@@ -4814,7 +4933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
         <v>128</v>
       </c>
@@ -4846,7 +4965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
         <v>129</v>
       </c>
@@ -4878,7 +4997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
         <v>130</v>
       </c>
@@ -4910,7 +5029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
         <v>131</v>
       </c>
@@ -4942,7 +5061,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
         <v>132</v>
       </c>
@@ -4974,10 +5093,10 @@
         <v>1</v>
       </c>
       <c r="K134" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
         <v>133</v>
       </c>
@@ -5009,7 +5128,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
         <v>134</v>
       </c>
@@ -5041,7 +5160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
         <v>135</v>
       </c>
@@ -5073,7 +5192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A138" s="1">
         <v>136</v>
       </c>
@@ -5105,7 +5224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
         <v>137</v>
       </c>
@@ -5137,7 +5256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A140" s="1">
         <v>138</v>
       </c>
@@ -5169,7 +5288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A141" s="1">
         <v>139</v>
       </c>
@@ -5201,7 +5320,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
         <v>140</v>
       </c>
@@ -5233,7 +5352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" s="1">
         <v>141</v>
       </c>
@@ -5265,7 +5384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
         <v>142</v>
       </c>
@@ -5297,7 +5416,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A145" s="1">
         <v>143</v>
       </c>
@@ -5329,7 +5448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
         <v>144</v>
       </c>
@@ -5361,7 +5480,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
         <v>145</v>
       </c>
@@ -5393,7 +5512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
         <v>146</v>
       </c>
@@ -5425,7 +5544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
         <v>147</v>
       </c>
@@ -5457,7 +5576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
         <v>148</v>
       </c>
@@ -5467,8 +5586,8 @@
       <c r="C150">
         <v>1</v>
       </c>
-      <c r="D150">
-        <v>0</v>
+      <c r="D150" s="8">
+        <v>1</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -5485,11 +5604,14 @@
       <c r="I150">
         <v>0</v>
       </c>
-      <c r="J150">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J150" s="8">
+        <v>2</v>
+      </c>
+      <c r="K150" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
         <v>149</v>
       </c>
@@ -5521,7 +5643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
         <v>150</v>
       </c>
@@ -5553,7 +5675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
         <v>151</v>
       </c>
@@ -5585,7 +5707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
         <v>152</v>
       </c>
@@ -5617,7 +5739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A155" s="1">
         <v>153</v>
       </c>
@@ -5649,7 +5771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A156" s="1">
         <v>154</v>
       </c>
@@ -5681,7 +5803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A157" s="1">
         <v>155</v>
       </c>
@@ -5713,7 +5835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A158" s="1">
         <v>156</v>
       </c>
@@ -5745,7 +5867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A159" s="1">
         <v>157</v>
       </c>
@@ -5777,7 +5899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A160" s="1">
         <v>158</v>
       </c>
@@ -5809,7 +5931,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A161" s="1">
         <v>159</v>
       </c>
@@ -5841,7 +5963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A162" s="1">
         <v>160</v>
       </c>
@@ -5873,7 +5995,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A163" s="1">
         <v>161</v>
       </c>
@@ -5905,7 +6027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A164" s="1">
         <v>162</v>
       </c>
@@ -5937,7 +6059,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A165" s="1">
         <v>163</v>
       </c>
@@ -5969,7 +6091,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A166" s="1">
         <v>164</v>
       </c>
@@ -6001,7 +6123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A167" s="1">
         <v>165</v>
       </c>
@@ -6033,7 +6155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A168" s="1">
         <v>166</v>
       </c>
@@ -6065,7 +6187,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A169" s="1">
         <v>167</v>
       </c>
@@ -6096,8 +6218,11 @@
       <c r="J169">
         <v>1</v>
       </c>
-    </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K169" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A170" s="1">
         <v>168</v>
       </c>
@@ -6129,7 +6254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A171" s="1">
         <v>169</v>
       </c>
@@ -6161,7 +6286,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A172" s="1">
         <v>170</v>
       </c>
@@ -6193,7 +6318,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" s="1">
         <v>171</v>
       </c>
@@ -6225,7 +6350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A174" s="1">
         <v>172</v>
       </c>
@@ -6257,7 +6382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A175" s="1">
         <v>173</v>
       </c>
@@ -6267,8 +6392,8 @@
       <c r="C175">
         <v>1</v>
       </c>
-      <c r="D175">
-        <v>0</v>
+      <c r="D175" s="8">
+        <v>3</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -6288,8 +6413,11 @@
       <c r="J175">
         <v>1</v>
       </c>
-    </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K175" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A176" s="1">
         <v>174</v>
       </c>
@@ -6320,8 +6448,11 @@
       <c r="J176">
         <v>1</v>
       </c>
-    </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K176" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A177" s="1">
         <v>175</v>
       </c>
@@ -6352,8 +6483,11 @@
       <c r="J177">
         <v>1</v>
       </c>
-    </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K177" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A178" s="1">
         <v>176</v>
       </c>
@@ -6385,7 +6519,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A179" s="1">
         <v>177</v>
       </c>
@@ -6417,7 +6551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A180" s="1">
         <v>178</v>
       </c>
@@ -6449,7 +6583,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A181" s="1">
         <v>179</v>
       </c>
@@ -6481,7 +6615,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A182" s="1">
         <v>180</v>
       </c>
@@ -6491,8 +6625,8 @@
       <c r="C182">
         <v>1</v>
       </c>
-      <c r="D182">
-        <v>0</v>
+      <c r="D182" s="8">
+        <v>1</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -6512,8 +6646,11 @@
       <c r="J182">
         <v>1</v>
       </c>
-    </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K182" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A183" s="1">
         <v>181</v>
       </c>
@@ -6545,7 +6682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A184" s="1">
         <v>182</v>
       </c>
@@ -6577,7 +6714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A185" s="1">
         <v>183</v>
       </c>
@@ -6609,7 +6746,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A186" s="1">
         <v>184</v>
       </c>
@@ -6641,7 +6778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A187" s="1">
         <v>185</v>
       </c>
@@ -6673,7 +6810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A188" s="1">
         <v>186</v>
       </c>
@@ -6705,7 +6842,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A189" s="1">
         <v>187</v>
       </c>
@@ -6737,7 +6874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A190" s="1">
         <v>188</v>
       </c>
@@ -6769,7 +6906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A191" s="1">
         <v>189</v>
       </c>
@@ -6801,7 +6938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A192" s="1">
         <v>190</v>
       </c>
@@ -6833,7 +6970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A193" s="1">
         <v>191</v>
       </c>
@@ -6865,7 +7002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A194" s="1">
         <v>192</v>
       </c>
@@ -6897,7 +7034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A195" s="1">
         <v>193</v>
       </c>
@@ -6908,7 +7045,7 @@
         <v>1</v>
       </c>
       <c r="D195" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E195">
         <v>0</v>
@@ -6929,10 +7066,10 @@
         <v>1</v>
       </c>
       <c r="K195" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A196" s="1">
         <v>194</v>
       </c>
@@ -6943,7 +7080,7 @@
         <v>1</v>
       </c>
       <c r="D196" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E196">
         <v>0</v>
@@ -6964,10 +7101,10 @@
         <v>1</v>
       </c>
       <c r="K196" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A197" s="1">
         <v>195</v>
       </c>
@@ -6999,7 +7136,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A198" s="1">
         <v>196</v>
       </c>
@@ -7031,7 +7168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A199" s="1">
         <v>197</v>
       </c>
@@ -7063,7 +7200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A200" s="1">
         <v>198</v>
       </c>
@@ -7074,7 +7211,7 @@
         <v>1</v>
       </c>
       <c r="D200" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E200">
         <v>0</v>
@@ -7095,10 +7232,10 @@
         <v>1</v>
       </c>
       <c r="K200" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A201" s="1">
         <v>199</v>
       </c>
@@ -7130,7 +7267,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A202" s="1">
         <v>200</v>
       </c>
@@ -7162,7 +7299,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A203" s="1">
         <v>201</v>
       </c>
@@ -7194,7 +7331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A204" s="1">
         <v>202</v>
       </c>
@@ -7226,7 +7363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A205" s="1">
         <v>203</v>
       </c>
@@ -7258,7 +7395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A206" s="1">
         <v>204</v>
       </c>
@@ -7290,7 +7427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A207" s="1">
         <v>205</v>
       </c>
@@ -7322,7 +7459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A208" s="1">
         <v>206</v>
       </c>
@@ -7354,7 +7491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A209" s="1">
         <v>207</v>
       </c>
@@ -7386,7 +7523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A210" s="1">
         <v>208</v>
       </c>
@@ -7418,7 +7555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A211" s="1">
         <v>209</v>
       </c>
@@ -7450,7 +7587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A212" s="1">
         <v>210</v>
       </c>
@@ -7482,7 +7619,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A213" s="1">
         <v>211</v>
       </c>
@@ -7514,7 +7651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A214" s="1">
         <v>212</v>
       </c>
@@ -7546,7 +7683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A215" s="1">
         <v>213</v>
       </c>
@@ -7578,7 +7715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A216" s="1">
         <v>214</v>
       </c>
@@ -7610,7 +7747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A217" s="1">
         <v>215</v>
       </c>
@@ -7642,7 +7779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A218" s="1">
         <v>216</v>
       </c>
@@ -7674,7 +7811,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A219" s="1">
         <v>217</v>
       </c>
@@ -7706,7 +7843,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A220" s="1">
         <v>218</v>
       </c>
@@ -7738,7 +7875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A221" s="1">
         <v>219</v>
       </c>
@@ -7770,7 +7907,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A222" s="1">
         <v>220</v>
       </c>
@@ -7802,7 +7939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A223" s="1">
         <v>221</v>
       </c>
@@ -7834,7 +7971,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A224" s="1">
         <v>222</v>
       </c>
@@ -7866,7 +8003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A225" s="1">
         <v>223</v>
       </c>
@@ -7898,7 +8035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A226" s="1">
         <v>224</v>
       </c>
@@ -7930,7 +8067,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A227" s="1">
         <v>225</v>
       </c>
@@ -7962,7 +8099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A228" s="1">
         <v>226</v>
       </c>
@@ -7994,7 +8131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A229" s="1">
         <v>227</v>
       </c>
@@ -8026,7 +8163,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A230" s="1">
         <v>228</v>
       </c>
@@ -8058,7 +8195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A231" s="1">
         <v>229</v>
       </c>
@@ -8090,7 +8227,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A232" s="1">
         <v>230</v>
       </c>
@@ -8122,7 +8259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A233" s="1">
         <v>231</v>
       </c>
@@ -8154,7 +8291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A234" s="1">
         <v>232</v>
       </c>
@@ -8186,7 +8323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A235" s="1">
         <v>233</v>
       </c>
@@ -8218,7 +8355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A236" s="1">
         <v>234</v>
       </c>
@@ -8250,7 +8387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A237" s="1">
         <v>235</v>
       </c>
@@ -8282,7 +8419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A238" s="1">
         <v>236</v>
       </c>
@@ -8314,7 +8451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A239" s="1">
         <v>237</v>
       </c>
@@ -8346,7 +8483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A240" s="1">
         <v>238</v>
       </c>
@@ -8378,7 +8515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A241" s="1">
         <v>239</v>
       </c>
@@ -8410,7 +8547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A242" s="1">
         <v>240</v>
       </c>
@@ -8442,7 +8579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A243" s="1">
         <v>241</v>
       </c>
@@ -8474,7 +8611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A244" s="1">
         <v>242</v>
       </c>
@@ -8506,7 +8643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A245" s="1">
         <v>243</v>
       </c>
@@ -8538,7 +8675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A246" s="1">
         <v>244</v>
       </c>
@@ -8570,7 +8707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A247" s="1">
         <v>245</v>
       </c>
@@ -8602,7 +8739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A248" s="1">
         <v>246</v>
       </c>
@@ -8634,7 +8771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A249" s="1">
         <v>247</v>
       </c>
@@ -8666,7 +8803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A250" s="1">
         <v>248</v>
       </c>
@@ -8698,7 +8835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A251" s="1">
         <v>249</v>
       </c>
@@ -8730,7 +8867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A252" s="1">
         <v>250</v>
       </c>
@@ -8762,7 +8899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A253" s="1">
         <v>251</v>
       </c>
@@ -8794,7 +8931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A254" s="1">
         <v>252</v>
       </c>
@@ -8826,7 +8963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A255" s="1">
         <v>253</v>
       </c>
@@ -8858,7 +8995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A256" s="1">
         <v>254</v>
       </c>
@@ -8890,7 +9027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A257" s="1">
         <v>255</v>
       </c>
@@ -8922,7 +9059,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="258" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A258" s="1">
         <v>256</v>
       </c>
@@ -8954,7 +9091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A259" s="1">
         <v>257</v>
       </c>
@@ -8986,7 +9123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A260" s="1">
         <v>258</v>
       </c>
@@ -9018,7 +9155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A261" s="1">
         <v>259</v>
       </c>
@@ -9050,7 +9187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A262" s="1">
         <v>260</v>
       </c>
@@ -9082,7 +9219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A263" s="1">
         <v>261</v>
       </c>
@@ -9114,7 +9251,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A264" s="1">
         <v>262</v>
       </c>
@@ -9146,7 +9283,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A265" s="1">
         <v>263</v>
       </c>
@@ -9178,7 +9315,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A266" s="1">
         <v>264</v>
       </c>
@@ -9210,7 +9347,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A267" s="1">
         <v>265</v>
       </c>
@@ -9242,7 +9379,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A268" s="1">
         <v>266</v>
       </c>
@@ -9274,7 +9411,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A269" s="1">
         <v>267</v>
       </c>
@@ -9285,7 +9422,7 @@
         <v>1</v>
       </c>
       <c r="D269" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E269">
         <v>1</v>
@@ -9306,10 +9443,10 @@
         <v>1</v>
       </c>
       <c r="K269" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="270" spans="1:11" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="270" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A270" s="1">
         <v>268</v>
       </c>
@@ -9341,7 +9478,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="271" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A271" s="1">
         <v>269</v>
       </c>
@@ -9352,7 +9489,7 @@
         <v>1</v>
       </c>
       <c r="D271" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E271">
         <v>0</v>
@@ -9373,10 +9510,10 @@
         <v>1</v>
       </c>
       <c r="K271" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="272" spans="1:11" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="272" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A272" s="1">
         <v>270</v>
       </c>
@@ -9408,7 +9545,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="273" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A273" s="1">
         <v>271</v>
       </c>
@@ -9440,7 +9577,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="274" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A274" s="1">
         <v>272</v>
       </c>
@@ -9472,7 +9609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A275" s="1">
         <v>273</v>
       </c>
@@ -9504,7 +9641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A276" s="1">
         <v>274</v>
       </c>
@@ -9536,7 +9673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A277" s="1">
         <v>275</v>
       </c>
@@ -9568,7 +9705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A278" s="1">
         <v>276</v>
       </c>
@@ -9600,7 +9737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A279" s="1">
         <v>277</v>
       </c>
@@ -9635,7 +9772,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="280" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A280" s="1">
         <v>278</v>
       </c>
@@ -9667,7 +9804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A281" s="1">
         <v>279</v>
       </c>
@@ -9699,7 +9836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A282" s="1">
         <v>280</v>
       </c>
@@ -9731,7 +9868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A283" s="1">
         <v>281</v>
       </c>
@@ -9763,7 +9900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A284" s="1">
         <v>282</v>
       </c>
@@ -9795,7 +9932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A285" s="1">
         <v>283</v>
       </c>
@@ -9827,7 +9964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A286" s="1">
         <v>284</v>
       </c>
@@ -9859,7 +9996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A287" s="1">
         <v>285</v>
       </c>
@@ -9891,7 +10028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A288" s="1">
         <v>286</v>
       </c>
@@ -9923,7 +10060,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A289" s="1">
         <v>287</v>
       </c>
@@ -9955,7 +10092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="290" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A290" s="1">
         <v>288</v>
       </c>
@@ -9966,7 +10103,7 @@
         <v>1</v>
       </c>
       <c r="D290" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E290">
         <v>1</v>
@@ -9987,10 +10124,10 @@
         <v>1</v>
       </c>
       <c r="K290" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A291" s="1">
         <v>289</v>
       </c>
@@ -10022,7 +10159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A292" s="1">
         <v>290</v>
       </c>
@@ -10033,7 +10170,7 @@
         <v>1</v>
       </c>
       <c r="D292" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E292">
         <v>1</v>
@@ -10054,10 +10191,10 @@
         <v>1</v>
       </c>
       <c r="K292" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A293" s="1">
         <v>291</v>
       </c>
@@ -10068,7 +10205,7 @@
         <v>1</v>
       </c>
       <c r="D293" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E293">
         <v>1</v>
@@ -10089,10 +10226,10 @@
         <v>1</v>
       </c>
       <c r="K293" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A294" s="1">
         <v>292</v>
       </c>
@@ -10124,7 +10261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A295" s="1">
         <v>293</v>
       </c>
@@ -10135,7 +10272,7 @@
         <v>1</v>
       </c>
       <c r="D295" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E295">
         <v>1</v>
@@ -10156,10 +10293,10 @@
         <v>1</v>
       </c>
       <c r="K295" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="296" spans="1:11" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A296" s="1">
         <v>294</v>
       </c>
@@ -10191,7 +10328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A297" s="1">
         <v>295</v>
       </c>
@@ -10223,7 +10360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A298" s="1">
         <v>296</v>
       </c>
@@ -10255,7 +10392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A299" s="1">
         <v>297</v>
       </c>
@@ -10287,7 +10424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A300" s="1">
         <v>298</v>
       </c>
@@ -10319,7 +10456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A301" s="1">
         <v>299</v>
       </c>
@@ -10351,7 +10488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A302" s="1">
         <v>300</v>
       </c>
@@ -10383,7 +10520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A303" s="1">
         <v>301</v>
       </c>
@@ -10415,7 +10552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A304" s="1">
         <v>302</v>
       </c>
@@ -10447,7 +10584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A305" s="1">
         <v>303</v>
       </c>
@@ -10479,7 +10616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A306" s="1">
         <v>304</v>
       </c>
@@ -10511,7 +10648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A307" s="1">
         <v>305</v>
       </c>
@@ -10543,7 +10680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A308" s="1">
         <v>306</v>
       </c>
@@ -10575,7 +10712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A309" s="1">
         <v>307</v>
       </c>
@@ -10607,7 +10744,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="310" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A310" s="1">
         <v>308</v>
       </c>
@@ -10639,7 +10776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A311" s="1">
         <v>309</v>
       </c>
@@ -10671,7 +10808,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="312" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A312" s="1">
         <v>310</v>
       </c>
@@ -10703,7 +10840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A313" s="1">
         <v>311</v>
       </c>
@@ -10735,7 +10872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A314" s="1">
         <v>312</v>
       </c>
@@ -10767,7 +10904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A315" s="1">
         <v>313</v>
       </c>
@@ -10799,7 +10936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A316" s="1">
         <v>314</v>
       </c>
@@ -10831,7 +10968,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="317" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A317" s="1">
         <v>315</v>
       </c>
@@ -10863,7 +11000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A318" s="1">
         <v>316</v>
       </c>
@@ -10895,7 +11032,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="319" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A319" s="1">
         <v>317</v>
       </c>
@@ -10927,7 +11064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A320" s="1">
         <v>318</v>
       </c>
@@ -10959,7 +11096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A321" s="1">
         <v>319</v>
       </c>
@@ -10991,7 +11128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A322" s="1">
         <v>320</v>
       </c>
@@ -11023,7 +11160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A323" s="1">
         <v>321</v>
       </c>
@@ -11055,7 +11192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A324" s="1">
         <v>322</v>
       </c>
@@ -11087,7 +11224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="325" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A325" s="1">
         <v>323</v>
       </c>
@@ -11119,7 +11256,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="326" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A326" s="1">
         <v>324</v>
       </c>
@@ -11151,7 +11288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="327" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A327" s="1">
         <v>325</v>
       </c>
@@ -11183,7 +11320,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="328" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A328" s="1">
         <v>326</v>
       </c>
@@ -11215,7 +11352,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="329" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A329" s="1">
         <v>327</v>
       </c>
@@ -11247,7 +11384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A330" s="1">
         <v>328</v>
       </c>
@@ -11279,7 +11416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A331" s="1">
         <v>329</v>
       </c>
@@ -11311,7 +11448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A332" s="1">
         <v>330</v>
       </c>
@@ -11343,7 +11480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A333" s="1">
         <v>331</v>
       </c>
@@ -11375,7 +11512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="334" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A334" s="1">
         <v>332</v>
       </c>
@@ -11407,7 +11544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A335" s="1">
         <v>333</v>
       </c>
@@ -11439,7 +11576,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A336" s="1">
         <v>334</v>
       </c>
@@ -11471,7 +11608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A337" s="1">
         <v>335</v>
       </c>
@@ -11503,7 +11640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A338" s="1">
         <v>336</v>
       </c>
@@ -11535,7 +11672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A339" s="1">
         <v>337</v>
       </c>
@@ -11567,7 +11704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A340" s="1">
         <v>338</v>
       </c>
@@ -11599,7 +11736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A341" s="1">
         <v>339</v>
       </c>
@@ -11631,7 +11768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A342" s="1">
         <v>340</v>
       </c>
@@ -11663,7 +11800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A343" s="1">
         <v>341</v>
       </c>
@@ -11695,7 +11832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A344" s="1">
         <v>342</v>
       </c>
@@ -11727,7 +11864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="345" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A345" s="1">
         <v>343</v>
       </c>
@@ -11759,10 +11896,10 @@
         <v>2</v>
       </c>
       <c r="K345" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="346" spans="1:11" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="346" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A346" s="1">
         <v>344</v>
       </c>
@@ -11794,7 +11931,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="347" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A347" s="1">
         <v>345</v>
       </c>
@@ -11826,7 +11963,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="348" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A348" s="1">
         <v>346</v>
       </c>
@@ -11858,7 +11995,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="349" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A349" s="1">
         <v>347</v>
       </c>
@@ -11890,10 +12027,10 @@
         <v>3</v>
       </c>
       <c r="K349" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="350" spans="1:11" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="350" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A350" s="1">
         <v>348</v>
       </c>
@@ -11925,7 +12062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="351" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A351" s="1">
         <v>349</v>
       </c>
@@ -11957,10 +12094,10 @@
         <v>1</v>
       </c>
       <c r="K351" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="352" spans="1:11" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="352" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A352" s="1">
         <v>350</v>
       </c>
@@ -11992,8 +12129,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="353" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A353" s="1">
+    <row r="353" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A353" s="7">
         <v>351</v>
       </c>
       <c r="B353">
@@ -12005,7 +12142,7 @@
       <c r="D353">
         <v>0</v>
       </c>
-      <c r="E353">
+      <c r="E353" s="8">
         <v>1</v>
       </c>
       <c r="F353">
@@ -12023,9 +12160,12 @@
       <c r="J353">
         <v>1</v>
       </c>
-    </row>
-    <row r="354" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A354" s="1">
+      <c r="K353" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="354" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A354" s="7">
         <v>352</v>
       </c>
       <c r="B354">
@@ -12037,14 +12177,14 @@
       <c r="D354">
         <v>0</v>
       </c>
-      <c r="E354">
-        <v>1</v>
+      <c r="E354" s="8">
+        <v>2</v>
       </c>
       <c r="F354">
         <v>1</v>
       </c>
-      <c r="G354">
-        <v>0</v>
+      <c r="G354" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H354">
         <v>0</v>
@@ -12055,9 +12195,12 @@
       <c r="J354">
         <v>1</v>
       </c>
-    </row>
-    <row r="355" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A355" s="1">
+      <c r="K354" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="355" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A355" s="7">
         <v>353</v>
       </c>
       <c r="B355">
@@ -12069,14 +12212,14 @@
       <c r="D355">
         <v>0</v>
       </c>
-      <c r="E355">
-        <v>1</v>
+      <c r="E355" s="8">
+        <v>2</v>
       </c>
       <c r="F355">
         <v>1</v>
       </c>
-      <c r="G355">
-        <v>0</v>
+      <c r="G355" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H355">
         <v>0</v>
@@ -12087,8 +12230,11 @@
       <c r="J355">
         <v>1</v>
       </c>
-    </row>
-    <row r="356" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K355" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="356" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A356" s="1">
         <v>354</v>
       </c>
@@ -12120,7 +12266,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="357" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A357" s="1">
         <v>355</v>
       </c>
@@ -12130,17 +12276,17 @@
       <c r="C357">
         <v>1</v>
       </c>
-      <c r="D357">
-        <v>2</v>
-      </c>
-      <c r="E357">
-        <v>1</v>
+      <c r="D357" s="8">
+        <v>3</v>
+      </c>
+      <c r="E357" s="8">
+        <v>2</v>
       </c>
       <c r="F357">
         <v>1</v>
       </c>
-      <c r="G357">
-        <v>0</v>
+      <c r="G357" s="8">
+        <v>3</v>
       </c>
       <c r="H357">
         <v>0</v>
@@ -12148,11 +12294,14 @@
       <c r="I357">
         <v>0</v>
       </c>
-      <c r="J357">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="358" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J357" s="8">
+        <v>4</v>
+      </c>
+      <c r="K357" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="358" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A358" s="1">
         <v>356</v>
       </c>
@@ -12184,7 +12333,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="359" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A359" s="1">
         <v>357</v>
       </c>
@@ -12216,7 +12365,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="360" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A360" s="1">
         <v>358</v>
       </c>
@@ -12229,14 +12378,14 @@
       <c r="D360">
         <v>0</v>
       </c>
-      <c r="E360">
-        <v>1</v>
+      <c r="E360" s="8">
+        <v>2</v>
       </c>
       <c r="F360">
         <v>1</v>
       </c>
-      <c r="G360">
-        <v>0</v>
+      <c r="G360" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H360">
         <v>0</v>
@@ -12247,8 +12396,11 @@
       <c r="J360">
         <v>1</v>
       </c>
-    </row>
-    <row r="361" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K360" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="361" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A361" s="1">
         <v>359</v>
       </c>
@@ -12280,7 +12432,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="362" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A362" s="1">
         <v>360</v>
       </c>
@@ -12312,7 +12464,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="363" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A363" s="1">
         <v>361</v>
       </c>
@@ -12325,14 +12477,14 @@
       <c r="D363">
         <v>0</v>
       </c>
-      <c r="E363">
-        <v>1</v>
+      <c r="E363" s="8">
+        <v>2</v>
       </c>
       <c r="F363">
         <v>1</v>
       </c>
-      <c r="G363">
-        <v>0</v>
+      <c r="G363" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H363">
         <v>0</v>
@@ -12343,8 +12495,11 @@
       <c r="J363">
         <v>1</v>
       </c>
-    </row>
-    <row r="364" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K363" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="364" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A364" s="1">
         <v>362</v>
       </c>
@@ -12376,7 +12531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="365" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A365" s="1">
         <v>363</v>
       </c>
@@ -12408,7 +12563,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="366" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A366" s="1">
         <v>364</v>
       </c>
@@ -12440,7 +12595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="367" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A367" s="1">
         <v>365</v>
       </c>
@@ -12450,8 +12605,8 @@
       <c r="C367">
         <v>1</v>
       </c>
-      <c r="D367">
-        <v>0</v>
+      <c r="D367" s="8" t="s">
+        <v>11</v>
       </c>
       <c r="E367">
         <v>1</v>
@@ -12471,8 +12626,11 @@
       <c r="J367">
         <v>1</v>
       </c>
-    </row>
-    <row r="368" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K367" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="368" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A368" s="1">
         <v>366</v>
       </c>
@@ -12504,7 +12662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A369" s="1">
         <v>367</v>
       </c>
@@ -12536,7 +12694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A370" s="1">
         <v>368</v>
       </c>
@@ -12568,7 +12726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A371" s="1">
         <v>369</v>
       </c>
@@ -12600,7 +12758,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="372" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A372" s="1">
         <v>370</v>
       </c>
@@ -12632,7 +12790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A373" s="1">
         <v>371</v>
       </c>
@@ -12664,7 +12822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="374" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A374" s="1">
         <v>372</v>
       </c>
@@ -12696,7 +12854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A375" s="1">
         <v>373</v>
       </c>
@@ -12728,7 +12886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A376" s="1">
         <v>374</v>
       </c>
@@ -12760,7 +12918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A377" s="1">
         <v>375</v>
       </c>
@@ -12792,7 +12950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A378" s="1">
         <v>376</v>
       </c>
@@ -12824,7 +12982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="379" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A379" s="1">
         <v>377</v>
       </c>
@@ -12856,7 +13014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A380" s="1">
         <v>378</v>
       </c>
@@ -12888,7 +13046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A381" s="1">
         <v>379</v>
       </c>
@@ -12920,7 +13078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="382" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A382" s="1">
         <v>380</v>
       </c>
@@ -12952,7 +13110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="383" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A383" s="1">
         <v>381</v>
       </c>
@@ -12984,7 +13142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="384" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A384" s="1">
         <v>382</v>
       </c>
@@ -13016,7 +13174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="385" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A385" s="1">
         <v>383</v>
       </c>
@@ -13048,7 +13206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="386" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A386" s="1">
         <v>384</v>
       </c>
@@ -13080,7 +13238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="387" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A387" s="1">
         <v>385</v>
       </c>
@@ -13112,7 +13270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="388" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A388" s="1">
         <v>386</v>
       </c>
@@ -13144,7 +13302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="389" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A389" s="1">
         <v>387</v>
       </c>
@@ -13176,7 +13334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="390" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A390" s="1">
         <v>388</v>
       </c>
@@ -13208,7 +13366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A391" s="1">
         <v>389</v>
       </c>
@@ -13240,7 +13398,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="392" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A392" s="1">
         <v>390</v>
       </c>
@@ -13272,7 +13430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="393" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A393" s="1">
         <v>391</v>
       </c>
@@ -13304,7 +13462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="394" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A394" s="1">
         <v>392</v>
       </c>
@@ -13336,7 +13494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="395" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A395" s="1">
         <v>393</v>
       </c>
@@ -13368,7 +13526,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="396" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A396" s="1">
         <v>394</v>
       </c>
@@ -13400,7 +13558,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="397" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A397" s="1">
         <v>395</v>
       </c>
@@ -13432,7 +13590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="398" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A398" s="1">
         <v>396</v>
       </c>
@@ -13440,7 +13598,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="399" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A399" s="1">
         <v>397</v>
       </c>
@@ -13448,7 +13606,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="400" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A400" s="1">
         <v>398</v>
       </c>
@@ -13456,7 +13614,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="401" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A401" s="1">
         <v>399</v>
       </c>
@@ -13464,7 +13622,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="402" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A402" s="1">
         <v>400</v>
       </c>

</xml_diff>

<commit_message>
[ADD] Data Labeling editing finished
</commit_message>
<xml_diff>
--- a/data/Suspension Data Labeling_We_Re_edit.xlsx
+++ b/data/Suspension Data Labeling_We_Re_edit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vulf/Git/Hub/Drop_wall_impact/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GITHUB\Drop_wall_impact\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA535CBE-B201-0B45-B4BE-3F43E7450248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B848D9E-756F-40B2-9C4A-C2C22B58C215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21600" yWindow="19460" windowWidth="21600" windowHeight="18940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Labels" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="88">
   <si>
     <t>Test #</t>
   </si>
@@ -265,12 +265,108 @@
   <si>
     <t>* Одна отсоединённая на виде сверху крупная капля</t>
   </si>
+  <si>
+    <t>*Брызг нет! Но капля оставляет след из частиц при сборе!</t>
+  </si>
+  <si>
+    <t>*Капля отделяется при окончании распространеня капли (и начале сбора)</t>
+  </si>
+  <si>
+    <t>*Брызг нет! Но есть начало формирования "зубьев"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* На виде спереди капля почти отделилась при распространении. На виде сверху - начало </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gear. Но потом, стекающая капля собрала их</t>
+    </r>
+  </si>
+  <si>
+    <t>*Брызг нет! Но есть отделение капель</t>
+  </si>
+  <si>
+    <t>* Отлетают крупные капли</t>
+  </si>
+  <si>
+    <t>*Брызг нет! Частицы остаются на подложке при стекании капли</t>
+  </si>
+  <si>
+    <t>* Разбрызгивание и отскок!</t>
+  </si>
+  <si>
+    <t>* Только одна капля отлетела в процессе расхождения. Остальное при сборе капли!</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* Отлетают три мелких капли. Начинает образовываться </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gear</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, но затем поглощается стекающей каплей</t>
+    </r>
+  </si>
+  <si>
+    <t>* Часть крупных капель отлетает при распространении капли, а часть при её сборе</t>
+  </si>
+  <si>
+    <t>* Множество крупных капель отсоединаются при распространении капли</t>
+  </si>
+  <si>
+    <t>* Разбрызгивания нет!</t>
+  </si>
+  <si>
+    <t>* Разбрызгивание есть. Отскока почти нет</t>
+  </si>
+  <si>
+    <t>* Есть разбрызгивание, есть разбиение капли при сборе, но вертикального отскока нет</t>
+  </si>
+  <si>
+    <t>* Разбрызгивание есть, разбиение капли при сборе есть. Вертикального отскока нет</t>
+  </si>
+  <si>
+    <t>* Разбрызгивание есть, разбиение капли при сборе есть (они собираются). Вертикального отскока нет</t>
+  </si>
+  <si>
+    <t>* Разбрызгивание есть!</t>
+  </si>
+  <si>
+    <t>* Есть разбрызгивание!</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -347,6 +443,23 @@
       <color rgb="FF000000"/>
       <name val="Calibri (Body)"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -389,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -412,6 +525,11 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,21 +833,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K402"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" customWidth="1"/>
-    <col min="7" max="7" width="20.5" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13.5" customWidth="1"/>
-    <col min="11" max="11" width="30.33203125" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" customWidth="1"/>
+    <col min="11" max="11" width="30.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="84" customHeight="1">
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
@@ -745,7 +863,7 @@
       <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -761,7 +879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="192" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="240">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -791,7 +909,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -802,7 +920,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -834,7 +952,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -866,7 +984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -898,7 +1016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -933,7 +1051,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -965,7 +1083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1000,7 +1118,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1035,7 +1153,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1070,7 +1188,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1102,7 +1220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1134,7 +1252,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1166,7 +1284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1198,7 +1316,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1230,7 +1348,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1262,7 +1380,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1297,7 +1415,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -1332,7 +1450,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1367,7 +1485,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1402,7 +1520,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1434,7 +1552,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1466,7 +1584,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1498,7 +1616,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1530,7 +1648,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1562,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1594,7 +1712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1629,7 +1747,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1664,7 +1782,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1696,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -1728,7 +1846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -1760,7 +1878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1795,7 +1913,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -1827,7 +1945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -1859,7 +1977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -1891,7 +2009,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -1923,7 +2041,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -1955,7 +2073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -1987,7 +2105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -2019,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -2051,7 +2169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -2083,7 +2201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -2115,7 +2233,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -2147,7 +2265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -2179,7 +2297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -2211,7 +2329,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -2243,7 +2361,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -2275,7 +2393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -2307,7 +2425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -2339,7 +2457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -2374,7 +2492,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -2406,7 +2524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -2441,7 +2559,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -2473,7 +2591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -2508,7 +2626,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -2543,7 +2661,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11">
       <c r="A57" s="1">
         <v>55</v>
       </c>
@@ -2575,7 +2693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11">
       <c r="A58" s="1">
         <v>56</v>
       </c>
@@ -2610,7 +2728,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11">
       <c r="A59" s="1">
         <v>57</v>
       </c>
@@ -2642,7 +2760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11">
       <c r="A60" s="1">
         <v>58</v>
       </c>
@@ -2674,7 +2792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11">
       <c r="A61" s="1">
         <v>59</v>
       </c>
@@ -2709,7 +2827,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11">
       <c r="A62" s="1">
         <v>60</v>
       </c>
@@ -2741,7 +2859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11">
       <c r="A63" s="1">
         <v>61</v>
       </c>
@@ -2773,7 +2891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11">
       <c r="A64" s="1">
         <v>62</v>
       </c>
@@ -2805,7 +2923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11">
       <c r="A65" s="1">
         <v>63</v>
       </c>
@@ -2840,7 +2958,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -2872,7 +2990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -2904,7 +3022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -2936,7 +3054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11">
       <c r="A69" s="1">
         <v>67</v>
       </c>
@@ -2968,7 +3086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11">
       <c r="A70" s="1">
         <v>68</v>
       </c>
@@ -3000,7 +3118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -3035,7 +3153,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -3070,7 +3188,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -3102,7 +3220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11">
       <c r="A74" s="1">
         <v>72</v>
       </c>
@@ -3134,7 +3252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -3166,7 +3284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11">
       <c r="A76" s="1">
         <v>74</v>
       </c>
@@ -3198,7 +3316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -3230,7 +3348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11">
       <c r="A78" s="1">
         <v>76</v>
       </c>
@@ -3262,7 +3380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11">
       <c r="A79" s="1">
         <v>77</v>
       </c>
@@ -3297,7 +3415,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11">
       <c r="A80" s="1">
         <v>78</v>
       </c>
@@ -3329,7 +3447,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11">
       <c r="A81" s="1">
         <v>79</v>
       </c>
@@ -3364,7 +3482,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11">
       <c r="A82" s="1">
         <v>80</v>
       </c>
@@ -3396,7 +3514,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:11">
       <c r="A83" s="1">
         <v>81</v>
       </c>
@@ -3428,7 +3546,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11">
       <c r="A84" s="1">
         <v>82</v>
       </c>
@@ -3460,7 +3578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11">
       <c r="A85" s="1">
         <v>83</v>
       </c>
@@ -3492,7 +3610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11">
       <c r="A86" s="1">
         <v>84</v>
       </c>
@@ -3524,7 +3642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11">
       <c r="A87" s="1">
         <v>85</v>
       </c>
@@ -3556,7 +3674,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11">
       <c r="A88" s="1">
         <v>86</v>
       </c>
@@ -3588,7 +3706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11">
       <c r="A89" s="1">
         <v>87</v>
       </c>
@@ -3620,7 +3738,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11">
       <c r="A90" s="1">
         <v>88</v>
       </c>
@@ -3652,7 +3770,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11">
       <c r="A91" s="1">
         <v>89</v>
       </c>
@@ -3684,7 +3802,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11">
       <c r="A92" s="1">
         <v>90</v>
       </c>
@@ -3716,7 +3834,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11">
       <c r="A93" s="1">
         <v>91</v>
       </c>
@@ -3751,7 +3869,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11">
       <c r="A94" s="1">
         <v>92</v>
       </c>
@@ -3783,7 +3901,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11">
       <c r="A95" s="1">
         <v>93</v>
       </c>
@@ -3818,7 +3936,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11">
       <c r="A96" s="1">
         <v>94</v>
       </c>
@@ -3853,7 +3971,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11">
       <c r="A97" s="1">
         <v>95</v>
       </c>
@@ -3888,7 +4006,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11">
       <c r="A98" s="1">
         <v>96</v>
       </c>
@@ -3920,7 +4038,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11">
       <c r="A99" s="1">
         <v>97</v>
       </c>
@@ -3952,7 +4070,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11">
       <c r="A100" s="1">
         <v>98</v>
       </c>
@@ -3984,7 +4102,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11">
       <c r="A101" s="1">
         <v>99</v>
       </c>
@@ -4016,7 +4134,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:11">
       <c r="A102" s="1">
         <v>100</v>
       </c>
@@ -4048,7 +4166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:11">
       <c r="A103" s="1">
         <v>101</v>
       </c>
@@ -4080,7 +4198,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:11">
       <c r="A104" s="1">
         <v>102</v>
       </c>
@@ -4093,8 +4211,8 @@
       <c r="D104" t="s">
         <v>11</v>
       </c>
-      <c r="E104">
-        <v>1</v>
+      <c r="E104" s="4">
+        <v>2</v>
       </c>
       <c r="F104">
         <v>2</v>
@@ -4102,7 +4220,7 @@
       <c r="G104">
         <v>3</v>
       </c>
-      <c r="H104">
+      <c r="H104" s="12">
         <v>1</v>
       </c>
       <c r="I104">
@@ -4111,8 +4229,11 @@
       <c r="J104" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K104" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11">
       <c r="A105" s="1">
         <v>103</v>
       </c>
@@ -4144,7 +4265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11">
       <c r="A106" s="1">
         <v>104</v>
       </c>
@@ -4176,7 +4297,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11">
       <c r="A107" s="1">
         <v>105</v>
       </c>
@@ -4208,7 +4329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11">
       <c r="A108" s="1">
         <v>106</v>
       </c>
@@ -4240,7 +4361,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:11">
       <c r="A109" s="1">
         <v>107</v>
       </c>
@@ -4272,7 +4393,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:11">
       <c r="A110" s="1">
         <v>108</v>
       </c>
@@ -4304,7 +4425,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:11">
       <c r="A111" s="1">
         <v>109</v>
       </c>
@@ -4336,7 +4457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:11">
       <c r="A112" s="1">
         <v>110</v>
       </c>
@@ -4368,7 +4489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:11">
       <c r="A113" s="1">
         <v>111</v>
       </c>
@@ -4400,7 +4521,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:11">
       <c r="A114" s="1">
         <v>112</v>
       </c>
@@ -4432,7 +4553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:11">
       <c r="A115" s="1">
         <v>113</v>
       </c>
@@ -4464,7 +4585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:11">
       <c r="A116" s="1">
         <v>114</v>
       </c>
@@ -4496,7 +4617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:11">
       <c r="A117" s="1">
         <v>115</v>
       </c>
@@ -4528,7 +4649,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:11">
       <c r="A118" s="1">
         <v>116</v>
       </c>
@@ -4560,7 +4681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:11">
       <c r="A119" s="1">
         <v>117</v>
       </c>
@@ -4595,7 +4716,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:11">
       <c r="A120" s="1">
         <v>118</v>
       </c>
@@ -4630,7 +4751,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:11">
       <c r="A121" s="1">
         <v>119</v>
       </c>
@@ -4665,7 +4786,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:11">
       <c r="A122" s="1">
         <v>120</v>
       </c>
@@ -4700,7 +4821,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:11">
       <c r="A123" s="1">
         <v>121</v>
       </c>
@@ -4735,7 +4856,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:11">
       <c r="A124" s="1">
         <v>122</v>
       </c>
@@ -4767,7 +4888,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:11">
       <c r="A125" s="1">
         <v>123</v>
       </c>
@@ -4799,7 +4920,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:11">
       <c r="A126" s="1">
         <v>124</v>
       </c>
@@ -4831,7 +4952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:11">
       <c r="A127" s="1">
         <v>125</v>
       </c>
@@ -4866,7 +4987,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:11">
       <c r="A128" s="1">
         <v>126</v>
       </c>
@@ -4901,7 +5022,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11">
       <c r="A129" s="1">
         <v>127</v>
       </c>
@@ -4933,7 +5054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11">
       <c r="A130" s="1">
         <v>128</v>
       </c>
@@ -4965,7 +5086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11">
       <c r="A131" s="1">
         <v>129</v>
       </c>
@@ -4997,7 +5118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11">
       <c r="A132" s="1">
         <v>130</v>
       </c>
@@ -5029,7 +5150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11">
       <c r="A133" s="1">
         <v>131</v>
       </c>
@@ -5061,7 +5182,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11">
       <c r="A134" s="1">
         <v>132</v>
       </c>
@@ -5096,7 +5217,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11">
       <c r="A135" s="1">
         <v>133</v>
       </c>
@@ -5128,7 +5249,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:11">
       <c r="A136" s="1">
         <v>134</v>
       </c>
@@ -5160,7 +5281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11">
       <c r="A137" s="1">
         <v>135</v>
       </c>
@@ -5192,7 +5313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11">
       <c r="A138" s="1">
         <v>136</v>
       </c>
@@ -5224,7 +5345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11">
       <c r="A139" s="1">
         <v>137</v>
       </c>
@@ -5256,7 +5377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11">
       <c r="A140" s="1">
         <v>138</v>
       </c>
@@ -5288,7 +5409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11">
       <c r="A141" s="1">
         <v>139</v>
       </c>
@@ -5320,7 +5441,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:11">
       <c r="A142" s="1">
         <v>140</v>
       </c>
@@ -5352,7 +5473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:11">
       <c r="A143" s="1">
         <v>141</v>
       </c>
@@ -5384,7 +5505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:11">
       <c r="A144" s="1">
         <v>142</v>
       </c>
@@ -5416,7 +5537,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:11">
       <c r="A145" s="1">
         <v>143</v>
       </c>
@@ -5448,7 +5569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:11">
       <c r="A146" s="1">
         <v>144</v>
       </c>
@@ -5480,7 +5601,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:11">
       <c r="A147" s="1">
         <v>145</v>
       </c>
@@ -5512,7 +5633,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:11">
       <c r="A148" s="1">
         <v>146</v>
       </c>
@@ -5544,7 +5665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:11">
       <c r="A149" s="1">
         <v>147</v>
       </c>
@@ -5576,7 +5697,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:11">
       <c r="A150" s="1">
         <v>148</v>
       </c>
@@ -5611,7 +5732,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:11">
       <c r="A151" s="1">
         <v>149</v>
       </c>
@@ -5643,7 +5764,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:11">
       <c r="A152" s="1">
         <v>150</v>
       </c>
@@ -5675,7 +5796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:11">
       <c r="A153" s="1">
         <v>151</v>
       </c>
@@ -5707,7 +5828,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:11">
       <c r="A154" s="1">
         <v>152</v>
       </c>
@@ -5739,7 +5860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:11">
       <c r="A155" s="1">
         <v>153</v>
       </c>
@@ -5771,7 +5892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:11">
       <c r="A156" s="1">
         <v>154</v>
       </c>
@@ -5803,7 +5924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:11">
       <c r="A157" s="1">
         <v>155</v>
       </c>
@@ -5835,7 +5956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:11">
       <c r="A158" s="1">
         <v>156</v>
       </c>
@@ -5867,7 +5988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:11">
       <c r="A159" s="1">
         <v>157</v>
       </c>
@@ -5899,7 +6020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:11">
       <c r="A160" s="1">
         <v>158</v>
       </c>
@@ -5931,7 +6052,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:11">
       <c r="A161" s="1">
         <v>159</v>
       </c>
@@ -5963,7 +6084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:11">
       <c r="A162" s="1">
         <v>160</v>
       </c>
@@ -5976,16 +6097,16 @@
       <c r="D162" t="s">
         <v>11</v>
       </c>
-      <c r="E162">
-        <v>1</v>
+      <c r="E162" s="4">
+        <v>2</v>
       </c>
       <c r="F162">
         <v>2</v>
       </c>
-      <c r="G162">
-        <v>0</v>
-      </c>
-      <c r="H162">
+      <c r="G162" s="4">
+        <v>4</v>
+      </c>
+      <c r="H162" s="12">
         <v>1</v>
       </c>
       <c r="I162">
@@ -5994,8 +6115,11 @@
       <c r="J162" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K162" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11">
       <c r="A163" s="1">
         <v>161</v>
       </c>
@@ -6027,7 +6151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:11">
       <c r="A164" s="1">
         <v>162</v>
       </c>
@@ -6059,7 +6183,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:11">
       <c r="A165" s="1">
         <v>163</v>
       </c>
@@ -6091,7 +6215,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:11">
       <c r="A166" s="1">
         <v>164</v>
       </c>
@@ -6123,7 +6247,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:11">
       <c r="A167" s="1">
         <v>165</v>
       </c>
@@ -6155,7 +6279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:11">
       <c r="A168" s="1">
         <v>166</v>
       </c>
@@ -6187,7 +6311,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:11">
       <c r="A169" s="1">
         <v>167</v>
       </c>
@@ -6222,7 +6346,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:11">
       <c r="A170" s="1">
         <v>168</v>
       </c>
@@ -6254,7 +6378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:11">
       <c r="A171" s="1">
         <v>169</v>
       </c>
@@ -6286,7 +6410,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:11">
       <c r="A172" s="1">
         <v>170</v>
       </c>
@@ -6299,16 +6423,16 @@
       <c r="D172" t="s">
         <v>11</v>
       </c>
-      <c r="E172">
-        <v>1</v>
+      <c r="E172" s="4">
+        <v>2</v>
       </c>
       <c r="F172">
         <v>2</v>
       </c>
-      <c r="G172">
-        <v>0</v>
-      </c>
-      <c r="H172">
+      <c r="G172" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H172" s="12">
         <v>1</v>
       </c>
       <c r="I172">
@@ -6317,8 +6441,11 @@
       <c r="J172" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K172" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11">
       <c r="A173" s="1">
         <v>171</v>
       </c>
@@ -6350,7 +6477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:11">
       <c r="A174" s="1">
         <v>172</v>
       </c>
@@ -6382,7 +6509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:11">
       <c r="A175" s="1">
         <v>173</v>
       </c>
@@ -6417,7 +6544,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:11">
       <c r="A176" s="1">
         <v>174</v>
       </c>
@@ -6452,7 +6579,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:11">
       <c r="A177" s="1">
         <v>175</v>
       </c>
@@ -6487,7 +6614,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:11">
       <c r="A178" s="1">
         <v>176</v>
       </c>
@@ -6519,7 +6646,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:11">
       <c r="A179" s="1">
         <v>177</v>
       </c>
@@ -6532,16 +6659,16 @@
       <c r="D179" t="s">
         <v>11</v>
       </c>
-      <c r="E179">
-        <v>1</v>
+      <c r="E179" s="4">
+        <v>2</v>
       </c>
       <c r="F179">
         <v>2</v>
       </c>
-      <c r="G179">
-        <v>0</v>
-      </c>
-      <c r="H179">
+      <c r="G179" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H179" s="12">
         <v>1</v>
       </c>
       <c r="I179">
@@ -6550,8 +6677,11 @@
       <c r="J179">
         <v>3</v>
       </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K179" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="180" spans="1:11">
       <c r="A180" s="1">
         <v>178</v>
       </c>
@@ -6583,7 +6713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11">
       <c r="A181" s="1">
         <v>179</v>
       </c>
@@ -6615,7 +6745,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11">
       <c r="A182" s="1">
         <v>180</v>
       </c>
@@ -6650,7 +6780,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:11">
       <c r="A183" s="1">
         <v>181</v>
       </c>
@@ -6682,7 +6812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11">
       <c r="A184" s="1">
         <v>182</v>
       </c>
@@ -6714,7 +6844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11">
       <c r="A185" s="1">
         <v>183</v>
       </c>
@@ -6746,7 +6876,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:11">
       <c r="A186" s="1">
         <v>184</v>
       </c>
@@ -6778,7 +6908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:11">
       <c r="A187" s="1">
         <v>185</v>
       </c>
@@ -6810,7 +6940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:11">
       <c r="A188" s="1">
         <v>186</v>
       </c>
@@ -6842,7 +6972,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:11">
       <c r="A189" s="1">
         <v>187</v>
       </c>
@@ -6874,7 +7004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:11">
       <c r="A190" s="1">
         <v>188</v>
       </c>
@@ -6906,7 +7036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:11">
       <c r="A191" s="1">
         <v>189</v>
       </c>
@@ -6938,7 +7068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:11">
       <c r="A192" s="1">
         <v>190</v>
       </c>
@@ -6970,7 +7100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:11">
       <c r="A193" s="1">
         <v>191</v>
       </c>
@@ -7002,7 +7132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:11">
       <c r="A194" s="1">
         <v>192</v>
       </c>
@@ -7034,7 +7164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:11">
       <c r="A195" s="1">
         <v>193</v>
       </c>
@@ -7069,7 +7199,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:11">
       <c r="A196" s="1">
         <v>194</v>
       </c>
@@ -7104,7 +7234,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:11">
       <c r="A197" s="1">
         <v>195</v>
       </c>
@@ -7136,7 +7266,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:11">
       <c r="A198" s="1">
         <v>196</v>
       </c>
@@ -7168,7 +7298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:11">
       <c r="A199" s="1">
         <v>197</v>
       </c>
@@ -7200,7 +7330,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:11">
       <c r="A200" s="1">
         <v>198</v>
       </c>
@@ -7235,7 +7365,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:11">
       <c r="A201" s="1">
         <v>199</v>
       </c>
@@ -7267,7 +7397,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:11">
       <c r="A202" s="1">
         <v>200</v>
       </c>
@@ -7299,7 +7429,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:11">
       <c r="A203" s="1">
         <v>201</v>
       </c>
@@ -7331,7 +7461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:11">
       <c r="A204" s="1">
         <v>202</v>
       </c>
@@ -7363,7 +7493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:11">
       <c r="A205" s="1">
         <v>203</v>
       </c>
@@ -7376,14 +7506,14 @@
       <c r="D205" t="s">
         <v>11</v>
       </c>
-      <c r="E205">
-        <v>1</v>
-      </c>
-      <c r="F205">
-        <v>1</v>
-      </c>
-      <c r="G205">
-        <v>0</v>
+      <c r="E205" s="4">
+        <v>2</v>
+      </c>
+      <c r="F205" s="4">
+        <v>2</v>
+      </c>
+      <c r="G205" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H205">
         <v>0</v>
@@ -7394,8 +7524,11 @@
       <c r="J205" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K205" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11">
       <c r="A206" s="1">
         <v>204</v>
       </c>
@@ -7426,8 +7559,11 @@
       <c r="J206">
         <v>2</v>
       </c>
-    </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K206" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11">
       <c r="A207" s="1">
         <v>205</v>
       </c>
@@ -7459,7 +7595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:11">
       <c r="A208" s="1">
         <v>206</v>
       </c>
@@ -7491,7 +7627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:11">
       <c r="A209" s="1">
         <v>207</v>
       </c>
@@ -7523,7 +7659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:11">
       <c r="A210" s="1">
         <v>208</v>
       </c>
@@ -7554,8 +7690,11 @@
       <c r="J210">
         <v>1</v>
       </c>
-    </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K210" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="211" spans="1:11">
       <c r="A211" s="1">
         <v>209</v>
       </c>
@@ -7586,8 +7725,11 @@
       <c r="J211">
         <v>1</v>
       </c>
-    </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K211" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="212" spans="1:11">
       <c r="A212" s="1">
         <v>210</v>
       </c>
@@ -7619,7 +7761,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:11">
       <c r="A213" s="1">
         <v>211</v>
       </c>
@@ -7651,7 +7793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:11">
       <c r="A214" s="1">
         <v>212</v>
       </c>
@@ -7683,7 +7825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:11">
       <c r="A215" s="1">
         <v>213</v>
       </c>
@@ -7715,7 +7857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:11">
       <c r="A216" s="1">
         <v>214</v>
       </c>
@@ -7747,7 +7889,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:11">
       <c r="A217" s="1">
         <v>215</v>
       </c>
@@ -7779,7 +7921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:11">
       <c r="A218" s="1">
         <v>216</v>
       </c>
@@ -7811,7 +7953,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:11">
       <c r="A219" s="1">
         <v>217</v>
       </c>
@@ -7843,7 +7985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:11">
       <c r="A220" s="1">
         <v>218</v>
       </c>
@@ -7875,7 +8017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:11">
       <c r="A221" s="1">
         <v>219</v>
       </c>
@@ -7907,7 +8049,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:11">
       <c r="A222" s="1">
         <v>220</v>
       </c>
@@ -7939,7 +8081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:11">
       <c r="A223" s="1">
         <v>221</v>
       </c>
@@ -7971,7 +8113,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:11">
       <c r="A224" s="1">
         <v>222</v>
       </c>
@@ -8003,7 +8145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:11">
       <c r="A225" s="1">
         <v>223</v>
       </c>
@@ -8035,7 +8177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:11">
       <c r="A226" s="1">
         <v>224</v>
       </c>
@@ -8066,8 +8208,11 @@
       <c r="J226" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K226" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="227" spans="1:11">
       <c r="A227" s="1">
         <v>225</v>
       </c>
@@ -8099,7 +8244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:11">
       <c r="A228" s="1">
         <v>226</v>
       </c>
@@ -8131,7 +8276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:11">
       <c r="A229" s="1">
         <v>227</v>
       </c>
@@ -8162,8 +8307,11 @@
       <c r="J229" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K229" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="230" spans="1:11">
       <c r="A230" s="1">
         <v>228</v>
       </c>
@@ -8195,7 +8343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:11">
       <c r="A231" s="1">
         <v>229</v>
       </c>
@@ -8226,8 +8374,11 @@
       <c r="J231" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K231" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="232" spans="1:11">
       <c r="A232" s="1">
         <v>230</v>
       </c>
@@ -8258,8 +8409,11 @@
       <c r="J232" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K232" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="233" spans="1:11">
       <c r="A233" s="1">
         <v>231</v>
       </c>
@@ -8291,7 +8445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:11">
       <c r="A234" s="1">
         <v>232</v>
       </c>
@@ -8323,7 +8477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:11">
       <c r="A235" s="1">
         <v>233</v>
       </c>
@@ -8355,7 +8509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:11">
       <c r="A236" s="1">
         <v>234</v>
       </c>
@@ -8387,7 +8541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:11">
       <c r="A237" s="1">
         <v>235</v>
       </c>
@@ -8419,7 +8573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:11">
       <c r="A238" s="1">
         <v>236</v>
       </c>
@@ -8451,7 +8605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:11">
       <c r="A239" s="1">
         <v>237</v>
       </c>
@@ -8483,7 +8637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:11">
       <c r="A240" s="1">
         <v>238</v>
       </c>
@@ -8515,7 +8669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10">
       <c r="A241" s="1">
         <v>239</v>
       </c>
@@ -8547,7 +8701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10">
       <c r="A242" s="1">
         <v>240</v>
       </c>
@@ -8579,7 +8733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10">
       <c r="A243" s="1">
         <v>241</v>
       </c>
@@ -8611,7 +8765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10">
       <c r="A244" s="1">
         <v>242</v>
       </c>
@@ -8643,7 +8797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10">
       <c r="A245" s="1">
         <v>243</v>
       </c>
@@ -8675,7 +8829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10">
       <c r="A246" s="1">
         <v>244</v>
       </c>
@@ -8707,7 +8861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10">
       <c r="A247" s="1">
         <v>245</v>
       </c>
@@ -8739,7 +8893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10">
       <c r="A248" s="1">
         <v>246</v>
       </c>
@@ -8771,7 +8925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10">
       <c r="A249" s="1">
         <v>247</v>
       </c>
@@ -8803,7 +8957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10">
       <c r="A250" s="1">
         <v>248</v>
       </c>
@@ -8835,7 +8989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10">
       <c r="A251" s="1">
         <v>249</v>
       </c>
@@ -8867,7 +9021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10">
       <c r="A252" s="1">
         <v>250</v>
       </c>
@@ -8899,7 +9053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10">
       <c r="A253" s="1">
         <v>251</v>
       </c>
@@ -8931,7 +9085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10">
       <c r="A254" s="1">
         <v>252</v>
       </c>
@@ -8963,7 +9117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10">
       <c r="A255" s="1">
         <v>253</v>
       </c>
@@ -8995,7 +9149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10">
       <c r="A256" s="1">
         <v>254</v>
       </c>
@@ -9027,7 +9181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:11">
       <c r="A257" s="1">
         <v>255</v>
       </c>
@@ -9037,11 +9191,11 @@
       <c r="C257">
         <v>1</v>
       </c>
-      <c r="D257" t="s">
-        <v>11</v>
-      </c>
-      <c r="E257">
-        <v>1</v>
+      <c r="D257" s="4">
+        <v>1</v>
+      </c>
+      <c r="E257" s="4">
+        <v>2</v>
       </c>
       <c r="F257">
         <v>2</v>
@@ -9058,8 +9212,11 @@
       <c r="J257" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="258" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K257" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="258" spans="1:11">
       <c r="A258" s="1">
         <v>256</v>
       </c>
@@ -9091,7 +9248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:11">
       <c r="A259" s="1">
         <v>257</v>
       </c>
@@ -9123,7 +9280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:11">
       <c r="A260" s="1">
         <v>258</v>
       </c>
@@ -9155,7 +9312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:11">
       <c r="A261" s="1">
         <v>259</v>
       </c>
@@ -9165,8 +9322,8 @@
       <c r="C261">
         <v>1</v>
       </c>
-      <c r="D261" t="s">
-        <v>11</v>
+      <c r="D261" s="4">
+        <v>3</v>
       </c>
       <c r="E261">
         <v>1</v>
@@ -9186,8 +9343,11 @@
       <c r="J261">
         <v>1</v>
       </c>
-    </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K261" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="262" spans="1:11">
       <c r="A262" s="1">
         <v>260</v>
       </c>
@@ -9219,7 +9379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:11">
       <c r="A263" s="1">
         <v>261</v>
       </c>
@@ -9251,7 +9411,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:11">
       <c r="A264" s="1">
         <v>262</v>
       </c>
@@ -9264,8 +9424,8 @@
       <c r="D264" t="s">
         <v>11</v>
       </c>
-      <c r="E264">
-        <v>1</v>
+      <c r="E264" s="4">
+        <v>2</v>
       </c>
       <c r="F264">
         <v>2</v>
@@ -9273,7 +9433,7 @@
       <c r="G264" t="s">
         <v>11</v>
       </c>
-      <c r="H264">
+      <c r="H264" s="12">
         <v>1</v>
       </c>
       <c r="I264">
@@ -9282,8 +9442,11 @@
       <c r="J264" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K264" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="265" spans="1:11">
       <c r="A265" s="1">
         <v>263</v>
       </c>
@@ -9315,7 +9478,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:11">
       <c r="A266" s="1">
         <v>264</v>
       </c>
@@ -9346,8 +9509,11 @@
       <c r="J266" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K266" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="267" spans="1:11">
       <c r="A267" s="1">
         <v>265</v>
       </c>
@@ -9379,7 +9545,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:11">
       <c r="A268" s="1">
         <v>266</v>
       </c>
@@ -9411,7 +9577,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:11">
       <c r="A269" s="1">
         <v>267</v>
       </c>
@@ -9446,7 +9612,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="270" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:11">
       <c r="A270" s="1">
         <v>268</v>
       </c>
@@ -9478,7 +9644,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="271" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:11">
       <c r="A271" s="1">
         <v>269</v>
       </c>
@@ -9513,7 +9679,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="272" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:11">
       <c r="A272" s="1">
         <v>270</v>
       </c>
@@ -9545,7 +9711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="273" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:11">
       <c r="A273" s="1">
         <v>271</v>
       </c>
@@ -9577,7 +9743,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="274" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:11">
       <c r="A274" s="1">
         <v>272</v>
       </c>
@@ -9608,8 +9774,11 @@
       <c r="J274">
         <v>1</v>
       </c>
-    </row>
-    <row r="275" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K274" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="275" spans="1:11">
       <c r="A275" s="1">
         <v>273</v>
       </c>
@@ -9622,14 +9791,14 @@
       <c r="D275">
         <v>0</v>
       </c>
-      <c r="E275">
-        <v>1</v>
+      <c r="E275" s="4">
+        <v>2</v>
       </c>
       <c r="F275">
         <v>1</v>
       </c>
-      <c r="G275">
-        <v>0</v>
+      <c r="G275" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="H275">
         <v>0</v>
@@ -9640,8 +9809,11 @@
       <c r="J275">
         <v>1</v>
       </c>
-    </row>
-    <row r="276" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K275" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="276" spans="1:11">
       <c r="A276" s="1">
         <v>274</v>
       </c>
@@ -9672,8 +9844,11 @@
       <c r="J276">
         <v>1</v>
       </c>
-    </row>
-    <row r="277" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K276" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="277" spans="1:11">
       <c r="A277" s="1">
         <v>275</v>
       </c>
@@ -9705,7 +9880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:11">
       <c r="A278" s="1">
         <v>276</v>
       </c>
@@ -9737,7 +9912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:11">
       <c r="A279" s="1">
         <v>277</v>
       </c>
@@ -9772,7 +9947,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="280" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:11">
       <c r="A280" s="1">
         <v>278</v>
       </c>
@@ -9782,17 +9957,17 @@
       <c r="C280">
         <v>1</v>
       </c>
-      <c r="D280" t="s">
-        <v>11</v>
-      </c>
-      <c r="E280">
-        <v>1</v>
+      <c r="D280" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E280" s="4">
+        <v>2</v>
       </c>
       <c r="F280">
         <v>1</v>
       </c>
-      <c r="G280">
-        <v>0</v>
+      <c r="G280" s="4">
+        <v>4</v>
       </c>
       <c r="H280">
         <v>0</v>
@@ -9803,8 +9978,11 @@
       <c r="J280">
         <v>1</v>
       </c>
-    </row>
-    <row r="281" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K280" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="281" spans="1:11">
       <c r="A281" s="1">
         <v>279</v>
       </c>
@@ -9835,8 +10013,11 @@
       <c r="J281">
         <v>1</v>
       </c>
-    </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K281" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="282" spans="1:11">
       <c r="A282" s="1">
         <v>280</v>
       </c>
@@ -9867,8 +10048,11 @@
       <c r="J282">
         <v>1</v>
       </c>
-    </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K282" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="283" spans="1:11">
       <c r="A283" s="1">
         <v>281</v>
       </c>
@@ -9900,7 +10084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:11">
       <c r="A284" s="1">
         <v>282</v>
       </c>
@@ -9932,7 +10116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:11">
       <c r="A285" s="1">
         <v>283</v>
       </c>
@@ -9964,7 +10148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:11">
       <c r="A286" s="1">
         <v>284</v>
       </c>
@@ -9996,7 +10180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:11">
       <c r="A287" s="1">
         <v>285</v>
       </c>
@@ -10028,7 +10212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:11">
       <c r="A288" s="1">
         <v>286</v>
       </c>
@@ -10060,7 +10244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:11">
       <c r="A289" s="1">
         <v>287</v>
       </c>
@@ -10092,7 +10276,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="290" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:11">
       <c r="A290" s="1">
         <v>288</v>
       </c>
@@ -10127,7 +10311,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:11">
       <c r="A291" s="1">
         <v>289</v>
       </c>
@@ -10159,7 +10343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:11">
       <c r="A292" s="1">
         <v>290</v>
       </c>
@@ -10194,7 +10378,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:11">
       <c r="A293" s="1">
         <v>291</v>
       </c>
@@ -10229,7 +10413,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:11">
       <c r="A294" s="1">
         <v>292</v>
       </c>
@@ -10261,7 +10445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:11">
       <c r="A295" s="1">
         <v>293</v>
       </c>
@@ -10296,7 +10480,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="296" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:11">
       <c r="A296" s="1">
         <v>294</v>
       </c>
@@ -10328,7 +10512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:11">
       <c r="A297" s="1">
         <v>295</v>
       </c>
@@ -10360,7 +10544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:11">
       <c r="A298" s="1">
         <v>296</v>
       </c>
@@ -10392,7 +10576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:11">
       <c r="A299" s="1">
         <v>297</v>
       </c>
@@ -10424,7 +10608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:11">
       <c r="A300" s="1">
         <v>298</v>
       </c>
@@ -10456,7 +10640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:11">
       <c r="A301" s="1">
         <v>299</v>
       </c>
@@ -10487,8 +10671,11 @@
       <c r="J301">
         <v>1</v>
       </c>
-    </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K301" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="302" spans="1:11">
       <c r="A302" s="1">
         <v>300</v>
       </c>
@@ -10519,8 +10706,11 @@
       <c r="J302">
         <v>1</v>
       </c>
-    </row>
-    <row r="303" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K302" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="303" spans="1:11">
       <c r="A303" s="1">
         <v>301</v>
       </c>
@@ -10552,7 +10742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:11">
       <c r="A304" s="1">
         <v>302</v>
       </c>
@@ -10584,7 +10774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:11">
       <c r="A305" s="1">
         <v>303</v>
       </c>
@@ -10615,8 +10805,11 @@
       <c r="J305">
         <v>1</v>
       </c>
-    </row>
-    <row r="306" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K305" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="306" spans="1:11">
       <c r="A306" s="1">
         <v>304</v>
       </c>
@@ -10648,7 +10841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:11">
       <c r="A307" s="1">
         <v>305</v>
       </c>
@@ -10679,9 +10872,12 @@
       <c r="J307">
         <v>1</v>
       </c>
-    </row>
-    <row r="308" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A308" s="1">
+      <c r="K307" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="308" spans="1:11">
+      <c r="A308" s="10">
         <v>306</v>
       </c>
       <c r="B308">
@@ -10705,14 +10901,17 @@
       <c r="H308">
         <v>1</v>
       </c>
-      <c r="I308">
-        <v>1</v>
+      <c r="I308" s="4">
+        <v>3</v>
       </c>
       <c r="J308">
         <v>1</v>
       </c>
-    </row>
-    <row r="309" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K308" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="309" spans="1:11">
       <c r="A309" s="1">
         <v>307</v>
       </c>
@@ -10722,8 +10921,8 @@
       <c r="C309">
         <v>1</v>
       </c>
-      <c r="D309">
-        <v>2</v>
+      <c r="D309" s="4">
+        <v>3</v>
       </c>
       <c r="E309">
         <v>1</v>
@@ -10743,8 +10942,11 @@
       <c r="J309">
         <v>2</v>
       </c>
-    </row>
-    <row r="310" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K309" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="310" spans="1:11">
       <c r="A310" s="1">
         <v>308</v>
       </c>
@@ -10776,7 +10978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:11">
       <c r="A311" s="1">
         <v>309</v>
       </c>
@@ -10807,8 +11009,11 @@
       <c r="J311">
         <v>2</v>
       </c>
-    </row>
-    <row r="312" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K311" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="312" spans="1:11">
       <c r="A312" s="1">
         <v>310</v>
       </c>
@@ -10840,7 +11045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:11">
       <c r="A313" s="1">
         <v>311</v>
       </c>
@@ -10872,7 +11077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:11">
       <c r="A314" s="1">
         <v>312</v>
       </c>
@@ -10903,8 +11108,11 @@
       <c r="J314">
         <v>1</v>
       </c>
-    </row>
-    <row r="315" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K314" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="315" spans="1:11">
       <c r="A315" s="1">
         <v>313</v>
       </c>
@@ -10935,8 +11143,11 @@
       <c r="J315">
         <v>1</v>
       </c>
-    </row>
-    <row r="316" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K315" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="316" spans="1:11">
       <c r="A316" s="1">
         <v>314</v>
       </c>
@@ -10968,7 +11179,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="317" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:11">
       <c r="A317" s="1">
         <v>315</v>
       </c>
@@ -11000,7 +11211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:11">
       <c r="A318" s="1">
         <v>316</v>
       </c>
@@ -11032,7 +11243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="319" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:11">
       <c r="A319" s="1">
         <v>317</v>
       </c>
@@ -11064,7 +11275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:11">
       <c r="A320" s="1">
         <v>318</v>
       </c>
@@ -11096,7 +11307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:10">
       <c r="A321" s="1">
         <v>319</v>
       </c>
@@ -11128,7 +11339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:10">
       <c r="A322" s="1">
         <v>320</v>
       </c>
@@ -11160,7 +11371,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:10">
       <c r="A323" s="1">
         <v>321</v>
       </c>
@@ -11192,7 +11403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:10">
       <c r="A324" s="1">
         <v>322</v>
       </c>
@@ -11224,7 +11435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="325" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:10">
       <c r="A325" s="1">
         <v>323</v>
       </c>
@@ -11256,7 +11467,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="326" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:10">
       <c r="A326" s="1">
         <v>324</v>
       </c>
@@ -11288,7 +11499,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="327" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:10">
       <c r="A327" s="1">
         <v>325</v>
       </c>
@@ -11320,7 +11531,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="328" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:10">
       <c r="A328" s="1">
         <v>326</v>
       </c>
@@ -11352,7 +11563,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="329" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:10">
       <c r="A329" s="1">
         <v>327</v>
       </c>
@@ -11384,7 +11595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:10">
       <c r="A330" s="1">
         <v>328</v>
       </c>
@@ -11416,7 +11627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:10">
       <c r="A331" s="1">
         <v>329</v>
       </c>
@@ -11448,7 +11659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:10">
       <c r="A332" s="1">
         <v>330</v>
       </c>
@@ -11480,7 +11691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:10">
       <c r="A333" s="1">
         <v>331</v>
       </c>
@@ -11512,7 +11723,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="334" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:10">
       <c r="A334" s="1">
         <v>332</v>
       </c>
@@ -11544,7 +11755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:10">
       <c r="A335" s="1">
         <v>333</v>
       </c>
@@ -11576,7 +11787,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:10">
       <c r="A336" s="1">
         <v>334</v>
       </c>
@@ -11608,7 +11819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:11">
       <c r="A337" s="1">
         <v>335</v>
       </c>
@@ -11640,7 +11851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:11">
       <c r="A338" s="1">
         <v>336</v>
       </c>
@@ -11672,7 +11883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:11">
       <c r="A339" s="1">
         <v>337</v>
       </c>
@@ -11682,8 +11893,8 @@
       <c r="C339">
         <v>1</v>
       </c>
-      <c r="D339" t="s">
-        <v>11</v>
+      <c r="D339" s="4">
+        <v>0</v>
       </c>
       <c r="E339">
         <v>1</v>
@@ -11703,8 +11914,11 @@
       <c r="J339">
         <v>1</v>
       </c>
-    </row>
-    <row r="340" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K339" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="340" spans="1:11">
       <c r="A340" s="1">
         <v>338</v>
       </c>
@@ -11736,7 +11950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:11">
       <c r="A341" s="1">
         <v>339</v>
       </c>
@@ -11768,7 +11982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:11">
       <c r="A342" s="1">
         <v>340</v>
       </c>
@@ -11800,7 +12014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:11">
       <c r="A343" s="1">
         <v>341</v>
       </c>
@@ -11832,7 +12046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:11">
       <c r="A344" s="1">
         <v>342</v>
       </c>
@@ -11864,7 +12078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="345" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:11">
       <c r="A345" s="1">
         <v>343</v>
       </c>
@@ -11899,7 +12113,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="346" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:11">
       <c r="A346" s="1">
         <v>344</v>
       </c>
@@ -11931,7 +12145,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="347" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:11">
       <c r="A347" s="1">
         <v>345</v>
       </c>
@@ -11963,7 +12177,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="348" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:11">
       <c r="A348" s="1">
         <v>346</v>
       </c>
@@ -11995,7 +12209,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="349" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:11">
       <c r="A349" s="1">
         <v>347</v>
       </c>
@@ -12030,7 +12244,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="350" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:11">
       <c r="A350" s="1">
         <v>348</v>
       </c>
@@ -12062,7 +12276,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="351" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:11">
       <c r="A351" s="1">
         <v>349</v>
       </c>
@@ -12097,7 +12311,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="352" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:11">
       <c r="A352" s="1">
         <v>350</v>
       </c>
@@ -12129,7 +12343,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="353" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:11">
       <c r="A353" s="7">
         <v>351</v>
       </c>
@@ -12164,7 +12378,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="354" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:11">
       <c r="A354" s="7">
         <v>352</v>
       </c>
@@ -12199,7 +12413,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="355" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:11">
       <c r="A355" s="7">
         <v>353</v>
       </c>
@@ -12234,7 +12448,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="356" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:11">
       <c r="A356" s="1">
         <v>354</v>
       </c>
@@ -12266,7 +12480,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="357" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:11">
       <c r="A357" s="1">
         <v>355</v>
       </c>
@@ -12301,7 +12515,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="358" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:11">
       <c r="A358" s="1">
         <v>356</v>
       </c>
@@ -12333,7 +12547,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="359" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:11">
       <c r="A359" s="1">
         <v>357</v>
       </c>
@@ -12365,7 +12579,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="360" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:11">
       <c r="A360" s="1">
         <v>358</v>
       </c>
@@ -12400,7 +12614,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="361" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:11">
       <c r="A361" s="1">
         <v>359</v>
       </c>
@@ -12432,7 +12646,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="362" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:11">
       <c r="A362" s="1">
         <v>360</v>
       </c>
@@ -12464,7 +12678,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="363" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:11">
       <c r="A363" s="1">
         <v>361</v>
       </c>
@@ -12499,7 +12713,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="364" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:11">
       <c r="A364" s="1">
         <v>362</v>
       </c>
@@ -12531,7 +12745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="365" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:11">
       <c r="A365" s="1">
         <v>363</v>
       </c>
@@ -12563,7 +12777,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="366" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:11">
       <c r="A366" s="1">
         <v>364</v>
       </c>
@@ -12595,7 +12809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="367" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:11">
       <c r="A367" s="1">
         <v>365</v>
       </c>
@@ -12630,7 +12844,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="368" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:11">
       <c r="A368" s="1">
         <v>366</v>
       </c>
@@ -12662,7 +12876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="369" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:10">
       <c r="A369" s="1">
         <v>367</v>
       </c>
@@ -12694,7 +12908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="370" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:10">
       <c r="A370" s="1">
         <v>368</v>
       </c>
@@ -12726,7 +12940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="371" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:10">
       <c r="A371" s="1">
         <v>369</v>
       </c>
@@ -12758,7 +12972,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="372" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:10">
       <c r="A372" s="1">
         <v>370</v>
       </c>
@@ -12790,7 +13004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:10">
       <c r="A373" s="1">
         <v>371</v>
       </c>
@@ -12822,7 +13036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="374" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:10">
       <c r="A374" s="1">
         <v>372</v>
       </c>
@@ -12854,7 +13068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:10">
       <c r="A375" s="1">
         <v>373</v>
       </c>
@@ -12886,7 +13100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:10">
       <c r="A376" s="1">
         <v>374</v>
       </c>
@@ -12918,7 +13132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:10">
       <c r="A377" s="1">
         <v>375</v>
       </c>
@@ -12950,7 +13164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:10">
       <c r="A378" s="1">
         <v>376</v>
       </c>
@@ -12982,7 +13196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="379" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:10">
       <c r="A379" s="1">
         <v>377</v>
       </c>
@@ -13014,7 +13228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:10">
       <c r="A380" s="1">
         <v>378</v>
       </c>
@@ -13046,7 +13260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:10">
       <c r="A381" s="1">
         <v>379</v>
       </c>
@@ -13078,7 +13292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="382" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:10">
       <c r="A382" s="1">
         <v>380</v>
       </c>
@@ -13110,7 +13324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="383" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:10">
       <c r="A383" s="1">
         <v>381</v>
       </c>
@@ -13142,7 +13356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="384" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:10">
       <c r="A384" s="1">
         <v>382</v>
       </c>
@@ -13174,7 +13388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="385" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:10">
       <c r="A385" s="1">
         <v>383</v>
       </c>
@@ -13206,7 +13420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="386" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="386" spans="1:10">
       <c r="A386" s="1">
         <v>384</v>
       </c>
@@ -13238,7 +13452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="387" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="387" spans="1:10">
       <c r="A387" s="1">
         <v>385</v>
       </c>
@@ -13270,7 +13484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="388" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="388" spans="1:10">
       <c r="A388" s="1">
         <v>386</v>
       </c>
@@ -13302,7 +13516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="389" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="389" spans="1:10">
       <c r="A389" s="1">
         <v>387</v>
       </c>
@@ -13334,7 +13548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="390" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:10">
       <c r="A390" s="1">
         <v>388</v>
       </c>
@@ -13366,7 +13580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:10">
       <c r="A391" s="1">
         <v>389</v>
       </c>
@@ -13398,7 +13612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="392" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:10">
       <c r="A392" s="1">
         <v>390</v>
       </c>
@@ -13430,7 +13644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="393" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:10">
       <c r="A393" s="1">
         <v>391</v>
       </c>
@@ -13462,7 +13676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="394" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:10">
       <c r="A394" s="1">
         <v>392</v>
       </c>
@@ -13494,7 +13708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="395" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:10">
       <c r="A395" s="1">
         <v>393</v>
       </c>
@@ -13526,7 +13740,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="396" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:10">
       <c r="A396" s="1">
         <v>394</v>
       </c>
@@ -13558,7 +13772,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="397" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:10">
       <c r="A397" s="1">
         <v>395</v>
       </c>
@@ -13590,7 +13804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="398" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:10">
       <c r="A398" s="1">
         <v>396</v>
       </c>
@@ -13598,7 +13812,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="399" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:10">
       <c r="A399" s="1">
         <v>397</v>
       </c>
@@ -13606,7 +13820,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="400" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:10">
       <c r="A400" s="1">
         <v>398</v>
       </c>
@@ -13614,7 +13828,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="401" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:2">
       <c r="A401" s="1">
         <v>399</v>
       </c>
@@ -13622,7 +13836,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="402" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:2">
       <c r="A402" s="1">
         <v>400</v>
       </c>

</xml_diff>

<commit_message>
[ADD] Edit test 351 and modify README in notebooks
</commit_message>
<xml_diff>
--- a/data/Suspension Data Labeling_We_Re_edit.xlsx
+++ b/data/Suspension Data Labeling_We_Re_edit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GITHUB\Drop_wall_impact\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4389AFF6-F029-4717-9149-938030A99D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23BFA3A-B56D-4D30-977E-4D38A51436FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Labels" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="98">
   <si>
     <t>Test #</t>
   </si>
@@ -196,9 +196,6 @@
   </si>
   <si>
     <t>*Брызг и зубьев нет! На виде спереди остаются частицы на подложке. Вид сверху плохо интерпретируется</t>
-  </si>
-  <si>
-    <t>*Брызг и зубьев нет! Однако на виде сверху виднеются разрывы</t>
   </si>
   <si>
     <t xml:space="preserve">*Есть как крупные капли, так и сохранение частиц на подложке при сборе капли </t>
@@ -404,6 +401,9 @@
   </si>
   <si>
     <t>* Есть и разбрызгивание, и отделение капель при сборе основной. Одна капля летит вертикально вверх, расценено как отскок</t>
+  </si>
+  <si>
+    <t>*Брызг и зубьев нет! Однако на виде сверху виднеются разрывы. Обозначим их причиной частицы</t>
   </si>
 </sst>
 </file>
@@ -905,7 +905,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>1</v>
@@ -937,7 +937,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>17</v>
@@ -952,7 +952,7 @@
         <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>21</v>
@@ -2382,7 +2382,7 @@
         <v>10</v>
       </c>
       <c r="K46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2612,7 +2612,7 @@
         <v>1</v>
       </c>
       <c r="K53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -2880,7 +2880,7 @@
         <v>1</v>
       </c>
       <c r="K61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3206,7 +3206,7 @@
         <v>1</v>
       </c>
       <c r="K71" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -3241,7 +3241,7 @@
         <v>1</v>
       </c>
       <c r="K72" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3535,7 +3535,7 @@
         <v>1</v>
       </c>
       <c r="K81" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -3666,7 +3666,7 @@
         <v>4</v>
       </c>
       <c r="K85" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -4289,7 +4289,7 @@
         <v>10</v>
       </c>
       <c r="K104" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -4356,7 +4356,7 @@
         <v>5</v>
       </c>
       <c r="K106" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -4423,7 +4423,7 @@
         <v>10</v>
       </c>
       <c r="K108" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -4586,7 +4586,7 @@
         <v>10</v>
       </c>
       <c r="K113" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="114" spans="1:11">
@@ -4816,7 +4816,7 @@
         <v>1</v>
       </c>
       <c r="K120" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="121" spans="1:11">
@@ -5509,7 +5509,7 @@
         <v>10</v>
       </c>
       <c r="K141" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="142" spans="1:11">
@@ -5800,7 +5800,7 @@
         <v>2</v>
       </c>
       <c r="K150" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="151" spans="1:11">
@@ -5899,7 +5899,7 @@
         <v>10</v>
       </c>
       <c r="K153" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="154" spans="1:11">
@@ -6126,7 +6126,7 @@
         <v>10</v>
       </c>
       <c r="K160" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="161" spans="1:11">
@@ -6193,7 +6193,7 @@
         <v>10</v>
       </c>
       <c r="K162" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="163" spans="1:11">
@@ -6292,7 +6292,7 @@
         <v>10</v>
       </c>
       <c r="K165" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="166" spans="1:11">
@@ -6490,7 +6490,7 @@
         <v>2</v>
       </c>
       <c r="K171" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="172" spans="1:11">
@@ -6525,7 +6525,7 @@
         <v>10</v>
       </c>
       <c r="K172" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="173" spans="1:11">
@@ -6624,7 +6624,7 @@
         <v>1</v>
       </c>
       <c r="K175" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="176" spans="1:11">
@@ -6761,7 +6761,7 @@
         <v>3</v>
       </c>
       <c r="K179" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="180" spans="1:11">
@@ -6796,7 +6796,7 @@
         <v>3</v>
       </c>
       <c r="K180" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="181" spans="1:11">
@@ -6831,7 +6831,7 @@
         <v>6</v>
       </c>
       <c r="K181" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -6866,7 +6866,7 @@
         <v>1</v>
       </c>
       <c r="K182" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="183" spans="1:11">
@@ -6901,7 +6901,7 @@
         <v>5</v>
       </c>
       <c r="K183" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -7617,7 +7617,7 @@
         <v>10</v>
       </c>
       <c r="K205" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="206" spans="1:11">
@@ -7652,7 +7652,7 @@
         <v>2</v>
       </c>
       <c r="K206" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="207" spans="1:11">
@@ -7853,7 +7853,7 @@
         <v>10</v>
       </c>
       <c r="K212" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="213" spans="1:11">
@@ -8080,7 +8080,7 @@
         <v>10</v>
       </c>
       <c r="K219" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="220" spans="1:11">
@@ -8307,7 +8307,7 @@
         <v>10</v>
       </c>
       <c r="K226" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="227" spans="1:11">
@@ -8406,7 +8406,7 @@
         <v>10</v>
       </c>
       <c r="K229" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="230" spans="1:11">
@@ -8473,7 +8473,7 @@
         <v>10</v>
       </c>
       <c r="K231" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="232" spans="1:11">
@@ -8508,7 +8508,7 @@
         <v>10</v>
       </c>
       <c r="K232" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="233" spans="1:11">
@@ -8575,7 +8575,7 @@
         <v>1</v>
       </c>
       <c r="K234" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="235" spans="1:11">
@@ -8674,7 +8674,7 @@
         <v>1</v>
       </c>
       <c r="K237" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="238" spans="1:11">
@@ -8773,7 +8773,7 @@
         <v>1</v>
       </c>
       <c r="K240" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="241" spans="1:11">
@@ -8904,7 +8904,7 @@
         <v>1</v>
       </c>
       <c r="K244" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="245" spans="1:11">
@@ -9003,7 +9003,7 @@
         <v>1</v>
       </c>
       <c r="K247" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -9070,7 +9070,7 @@
         <v>1</v>
       </c>
       <c r="K249" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="250" spans="1:11">
@@ -9201,7 +9201,7 @@
         <v>1</v>
       </c>
       <c r="K253" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="254" spans="1:11">
@@ -9332,7 +9332,7 @@
         <v>10</v>
       </c>
       <c r="K257" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="258" spans="1:11">
@@ -9463,7 +9463,7 @@
         <v>1</v>
       </c>
       <c r="K261" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="262" spans="1:11">
@@ -9562,7 +9562,7 @@
         <v>10</v>
       </c>
       <c r="K264" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="265" spans="1:11">
@@ -9629,7 +9629,7 @@
         <v>10</v>
       </c>
       <c r="K266" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="267" spans="1:11">
@@ -9917,7 +9917,7 @@
         <v>1</v>
       </c>
       <c r="G275" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H275">
         <v>0</v>
@@ -9929,7 +9929,7 @@
         <v>1</v>
       </c>
       <c r="K275" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="276" spans="1:11">
@@ -9964,7 +9964,7 @@
         <v>1</v>
       </c>
       <c r="K276" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="277" spans="1:11">
@@ -10098,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="K280" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="281" spans="1:11">
@@ -10168,7 +10168,7 @@
         <v>1</v>
       </c>
       <c r="K282" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="283" spans="1:11">
@@ -10203,7 +10203,7 @@
         <v>1</v>
       </c>
       <c r="K283" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="284" spans="1:11">
@@ -10270,7 +10270,7 @@
         <v>1</v>
       </c>
       <c r="K285" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="286" spans="1:11">
@@ -10369,7 +10369,7 @@
         <v>3</v>
       </c>
       <c r="K288" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="289" spans="1:11">
@@ -10800,7 +10800,7 @@
         <v>1</v>
       </c>
       <c r="K301" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="302" spans="1:11">
@@ -10835,7 +10835,7 @@
         <v>1</v>
       </c>
       <c r="K302" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="303" spans="1:11">
@@ -10934,7 +10934,7 @@
         <v>1</v>
       </c>
       <c r="K305" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="306" spans="1:11">
@@ -11036,7 +11036,7 @@
         <v>1</v>
       </c>
       <c r="K308" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="309" spans="1:11">
@@ -11071,7 +11071,7 @@
         <v>2</v>
       </c>
       <c r="K309" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="310" spans="1:11">
@@ -11138,7 +11138,7 @@
         <v>2</v>
       </c>
       <c r="K311" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="312" spans="1:11">
@@ -11237,7 +11237,7 @@
         <v>1</v>
       </c>
       <c r="K314" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="315" spans="1:11">
@@ -11272,7 +11272,7 @@
         <v>1</v>
       </c>
       <c r="K315" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="316" spans="1:11">
@@ -12043,7 +12043,7 @@
         <v>1</v>
       </c>
       <c r="K339" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="340" spans="1:11">
@@ -12273,7 +12273,7 @@
         <v>10</v>
       </c>
       <c r="K346" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="347" spans="1:11">
@@ -12407,7 +12407,7 @@
         <v>10</v>
       </c>
       <c r="K350" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="351" spans="1:11">
@@ -12477,7 +12477,7 @@
         <v>10</v>
       </c>
       <c r="K352" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="353" spans="1:11">
@@ -12494,13 +12494,13 @@
         <v>0</v>
       </c>
       <c r="E353" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F353">
         <v>1</v>
       </c>
-      <c r="G353">
-        <v>0</v>
+      <c r="G353" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="H353">
         <v>0</v>
@@ -12512,7 +12512,7 @@
         <v>1</v>
       </c>
       <c r="K353" t="s">
-        <v>54</v>
+        <v>97</v>
       </c>
     </row>
     <row r="354" spans="1:11">
@@ -12535,7 +12535,7 @@
         <v>1</v>
       </c>
       <c r="G354" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H354">
         <v>0</v>
@@ -12570,7 +12570,7 @@
         <v>1</v>
       </c>
       <c r="G355" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H355">
         <v>0</v>
@@ -12617,7 +12617,7 @@
         <v>10</v>
       </c>
       <c r="K356" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="357" spans="1:11">
@@ -12652,7 +12652,7 @@
         <v>4</v>
       </c>
       <c r="K357" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="358" spans="1:11">
@@ -12739,7 +12739,7 @@
         <v>1</v>
       </c>
       <c r="G360" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H360">
         <v>0</v>
@@ -12838,7 +12838,7 @@
         <v>1</v>
       </c>
       <c r="G363" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H363">
         <v>0</v>
@@ -12981,7 +12981,7 @@
         <v>1</v>
       </c>
       <c r="K367" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="368" spans="1:11">

</xml_diff>